<commit_message>
Udated process_results.py and plot_cement from main branch
</commit_message>
<xml_diff>
--- a/dataCaseStudy_Cement/raw_results/tech_selection/Summary.xlsx
+++ b/dataCaseStudy_Cement/raw_results/tech_selection/Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE13"/>
+  <dimension ref="A1:AE22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1818,6 +1818,933 @@
       <c r="AE13" t="inlineStr">
         <is>
           <t>dataCaseStudy_Cement\raw_results\tech_selection\20260302184520_carbon_tax_150_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>69379515.18200323</v>
+      </c>
+      <c r="B14" t="n">
+        <v>12204845.78141507</v>
+      </c>
+      <c r="C14" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D14" t="n">
+        <v>36483821.36884278</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>48688667.15025785</v>
+      </c>
+      <c r="G14" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H14" t="n">
+        <v>7660091.856915521</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="n">
+        <v>7260733.901533453</v>
+      </c>
+      <c r="M14" t="n">
+        <v>69379515.18200323</v>
+      </c>
+      <c r="N14" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R14" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V14" t="n">
+        <v>6.889999866485596</v>
+      </c>
+      <c r="W14" t="n">
+        <v>69379515.18200323</v>
+      </c>
+      <c r="X14" t="n">
+        <v>69379515.18200323</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>carbon_tax_50_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260302225945_carbon_tax_50_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>75043365.08214331</v>
+      </c>
+      <c r="B15" t="n">
+        <v>12204845.78141507</v>
+      </c>
+      <c r="C15" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D15" t="n">
+        <v>36483821.36884278</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>48688667.15025785</v>
+      </c>
+      <c r="G15" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H15" t="n">
+        <v>13323941.7570556</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="n">
+        <v>7260733.901533453</v>
+      </c>
+      <c r="M15" t="n">
+        <v>75043365.08214331</v>
+      </c>
+      <c r="N15" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R15" t="n">
+        <v>0</v>
+      </c>
+      <c r="S15" t="n">
+        <v>0</v>
+      </c>
+      <c r="T15" t="n">
+        <v>0</v>
+      </c>
+      <c r="U15" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V15" t="n">
+        <v>15.8840000629425</v>
+      </c>
+      <c r="W15" t="n">
+        <v>75043365.08214331</v>
+      </c>
+      <c r="X15" t="n">
+        <v>75043365.08214331</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>carbon_tax_50_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260302230243_carbon_tax_50_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>80707214.98228344</v>
+      </c>
+      <c r="B16" t="n">
+        <v>12204845.78141507</v>
+      </c>
+      <c r="C16" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D16" t="n">
+        <v>36483821.36884278</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>48688667.15025785</v>
+      </c>
+      <c r="G16" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H16" t="n">
+        <v>18987791.65719574</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="n">
+        <v>7260733.901533453</v>
+      </c>
+      <c r="M16" t="n">
+        <v>80707214.98228344</v>
+      </c>
+      <c r="N16" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" t="n">
+        <v>0</v>
+      </c>
+      <c r="T16" t="n">
+        <v>0</v>
+      </c>
+      <c r="U16" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V16" t="n">
+        <v>5.67300009727478</v>
+      </c>
+      <c r="W16" t="n">
+        <v>80707214.98228344</v>
+      </c>
+      <c r="X16" t="n">
+        <v>80707214.98228344</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>carbon_tax_50_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260302230631_carbon_tax_50_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>86371064.88242361</v>
+      </c>
+      <c r="B17" t="n">
+        <v>12204845.78141507</v>
+      </c>
+      <c r="C17" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D17" t="n">
+        <v>36483821.36884278</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>48688667.15025785</v>
+      </c>
+      <c r="G17" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H17" t="n">
+        <v>24651641.5573359</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="n">
+        <v>7260733.901533453</v>
+      </c>
+      <c r="M17" t="n">
+        <v>86371064.88242361</v>
+      </c>
+      <c r="N17" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R17" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" t="n">
+        <v>0</v>
+      </c>
+      <c r="T17" t="n">
+        <v>0</v>
+      </c>
+      <c r="U17" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V17" t="n">
+        <v>5.842000007629395</v>
+      </c>
+      <c r="W17" t="n">
+        <v>86371064.88242361</v>
+      </c>
+      <c r="X17" t="n">
+        <v>86371064.88242361</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>carbon_tax_50_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260302230911_carbon_tax_50_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>76640249.08353668</v>
+      </c>
+      <c r="B18" t="n">
+        <v>12204845.78141507</v>
+      </c>
+      <c r="C18" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D18" t="n">
+        <v>36483821.36884278</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>48688667.15025785</v>
+      </c>
+      <c r="G18" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H18" t="n">
+        <v>7660091.856915521</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="n">
+        <v>14521467.80306691</v>
+      </c>
+      <c r="M18" t="n">
+        <v>76640249.08353668</v>
+      </c>
+      <c r="N18" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R18" t="n">
+        <v>0</v>
+      </c>
+      <c r="S18" t="n">
+        <v>0</v>
+      </c>
+      <c r="T18" t="n">
+        <v>0</v>
+      </c>
+      <c r="U18" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V18" t="n">
+        <v>14.37700009346008</v>
+      </c>
+      <c r="W18" t="n">
+        <v>76640249.08353668</v>
+      </c>
+      <c r="X18" t="n">
+        <v>76640249.08353668</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>carbon_tax_100_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE18" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260302231229_carbon_tax_100_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>82304098.98367676</v>
+      </c>
+      <c r="B19" t="n">
+        <v>12204845.78141507</v>
+      </c>
+      <c r="C19" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D19" t="n">
+        <v>36483821.36884278</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>48688667.15025785</v>
+      </c>
+      <c r="G19" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H19" t="n">
+        <v>13323941.7570556</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" t="n">
+        <v>14521467.80306691</v>
+      </c>
+      <c r="M19" t="n">
+        <v>82304098.98367676</v>
+      </c>
+      <c r="N19" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R19" t="n">
+        <v>0</v>
+      </c>
+      <c r="S19" t="n">
+        <v>0</v>
+      </c>
+      <c r="T19" t="n">
+        <v>0</v>
+      </c>
+      <c r="U19" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V19" t="n">
+        <v>4.296999931335449</v>
+      </c>
+      <c r="W19" t="n">
+        <v>82304098.98367676</v>
+      </c>
+      <c r="X19" t="n">
+        <v>82304098.98367676</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>carbon_tax_100_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE19" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260302231853_carbon_tax_100_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>87967948.8838169</v>
+      </c>
+      <c r="B20" t="n">
+        <v>12204845.78141507</v>
+      </c>
+      <c r="C20" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D20" t="n">
+        <v>36483821.36884278</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>48688667.15025785</v>
+      </c>
+      <c r="G20" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H20" t="n">
+        <v>18987791.65719574</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="n">
+        <v>14521467.80306691</v>
+      </c>
+      <c r="M20" t="n">
+        <v>87967948.8838169</v>
+      </c>
+      <c r="N20" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R20" t="n">
+        <v>0</v>
+      </c>
+      <c r="S20" t="n">
+        <v>0</v>
+      </c>
+      <c r="T20" t="n">
+        <v>0</v>
+      </c>
+      <c r="U20" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V20" t="n">
+        <v>7.796000003814697</v>
+      </c>
+      <c r="W20" t="n">
+        <v>87967948.8838169</v>
+      </c>
+      <c r="X20" t="n">
+        <v>87967948.8838169</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>carbon_tax_100_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE20" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260302233051_carbon_tax_100_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>93631798.78395706</v>
+      </c>
+      <c r="B21" t="n">
+        <v>12204845.78141507</v>
+      </c>
+      <c r="C21" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D21" t="n">
+        <v>36483821.36884278</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>48688667.15025785</v>
+      </c>
+      <c r="G21" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H21" t="n">
+        <v>24651641.5573359</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" t="n">
+        <v>14521467.80306691</v>
+      </c>
+      <c r="M21" t="n">
+        <v>93631798.78395706</v>
+      </c>
+      <c r="N21" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R21" t="n">
+        <v>0</v>
+      </c>
+      <c r="S21" t="n">
+        <v>0</v>
+      </c>
+      <c r="T21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U21" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V21" t="n">
+        <v>6.632999897003174</v>
+      </c>
+      <c r="W21" t="n">
+        <v>93631798.78395706</v>
+      </c>
+      <c r="X21" t="n">
+        <v>93631798.78395706</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>carbon_tax_100_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE21" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260302234706_carbon_tax_100_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>83900982.98507079</v>
+      </c>
+      <c r="B22" t="n">
+        <v>12204845.78141507</v>
+      </c>
+      <c r="C22" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D22" t="n">
+        <v>36483821.36884278</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="n">
+        <v>48688667.15025785</v>
+      </c>
+      <c r="G22" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H22" t="n">
+        <v>7660091.856915521</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" t="n">
+        <v>21782201.70460102</v>
+      </c>
+      <c r="M22" t="n">
+        <v>83900982.98507079</v>
+      </c>
+      <c r="N22" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R22" t="n">
+        <v>0</v>
+      </c>
+      <c r="S22" t="n">
+        <v>0</v>
+      </c>
+      <c r="T22" t="n">
+        <v>0</v>
+      </c>
+      <c r="U22" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V22" t="n">
+        <v>9.075000047683716</v>
+      </c>
+      <c r="W22" t="n">
+        <v>83900982.98507079</v>
+      </c>
+      <c r="X22" t="n">
+        <v>83900982.98507079</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>carbon_tax_150_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE22" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260303000733_carbon_tax_150_el_price_50</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
results cement tech selection
</commit_message>
<xml_diff>
--- a/dataCaseStudy_Cement/raw_results/tech_selection/Summary.xlsx
+++ b/dataCaseStudy_Cement/raw_results/tech_selection/Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE22"/>
+  <dimension ref="A1:AE38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2745,6 +2745,1654 @@
       <c r="AE22" t="inlineStr">
         <is>
           <t>dataCaseStudy_Cement\raw_results\tech_selection\20260303000733_carbon_tax_150_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>69379515.18200326</v>
+      </c>
+      <c r="B23" t="n">
+        <v>12204845.78141508</v>
+      </c>
+      <c r="C23" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D23" t="n">
+        <v>36483821.3688428</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="n">
+        <v>48688667.15025788</v>
+      </c>
+      <c r="G23" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H23" t="n">
+        <v>7660091.856915521</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" t="n">
+        <v>7260733.901533453</v>
+      </c>
+      <c r="M23" t="n">
+        <v>69379515.18200326</v>
+      </c>
+      <c r="N23" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R23" t="n">
+        <v>0</v>
+      </c>
+      <c r="S23" t="n">
+        <v>0</v>
+      </c>
+      <c r="T23" t="n">
+        <v>0</v>
+      </c>
+      <c r="U23" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V23" t="n">
+        <v>8.654000043869019</v>
+      </c>
+      <c r="W23" t="n">
+        <v>69287006.76656619</v>
+      </c>
+      <c r="X23" t="n">
+        <v>69379515.18200326</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>92508.41543707252</v>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC23" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>carbon_tax_50_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE23" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308181035_carbon_tax_50_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>75043365.08214334</v>
+      </c>
+      <c r="B24" t="n">
+        <v>12204845.78141508</v>
+      </c>
+      <c r="C24" t="n">
+        <v>5770022.273296408</v>
+      </c>
+      <c r="D24" t="n">
+        <v>36483821.3688428</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="n">
+        <v>48688667.15025788</v>
+      </c>
+      <c r="G24" t="n">
+        <v>5770022.273296408</v>
+      </c>
+      <c r="H24" t="n">
+        <v>13323941.7570556</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" t="n">
+        <v>7260733.901533453</v>
+      </c>
+      <c r="M24" t="n">
+        <v>75043365.08214334</v>
+      </c>
+      <c r="N24" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O24" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R24" t="n">
+        <v>0</v>
+      </c>
+      <c r="S24" t="n">
+        <v>0</v>
+      </c>
+      <c r="T24" t="n">
+        <v>0</v>
+      </c>
+      <c r="U24" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V24" t="n">
+        <v>7.187999963760376</v>
+      </c>
+      <c r="W24" t="n">
+        <v>74899775.70983292</v>
+      </c>
+      <c r="X24" t="n">
+        <v>75043365.08214334</v>
+      </c>
+      <c r="Y24" t="n">
+        <v>143589.3723104149</v>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>carbon_tax_50_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE24" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308181423_carbon_tax_50_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>80707214.98228347</v>
+      </c>
+      <c r="B25" t="n">
+        <v>12204845.78141508</v>
+      </c>
+      <c r="C25" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D25" t="n">
+        <v>36483821.3688428</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="n">
+        <v>48688667.15025788</v>
+      </c>
+      <c r="G25" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H25" t="n">
+        <v>18987791.65719574</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" t="n">
+        <v>7260733.901533453</v>
+      </c>
+      <c r="M25" t="n">
+        <v>80707214.98228347</v>
+      </c>
+      <c r="N25" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O25" t="n">
+        <v>0</v>
+      </c>
+      <c r="P25" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R25" t="n">
+        <v>0</v>
+      </c>
+      <c r="S25" t="n">
+        <v>0</v>
+      </c>
+      <c r="T25" t="n">
+        <v>0</v>
+      </c>
+      <c r="U25" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V25" t="n">
+        <v>6.769000053405762</v>
+      </c>
+      <c r="W25" t="n">
+        <v>80563625.60997264</v>
+      </c>
+      <c r="X25" t="n">
+        <v>80707214.98228347</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>143589.3723108321</v>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD25" t="inlineStr">
+        <is>
+          <t>carbon_tax_50_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE25" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308181751_carbon_tax_50_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>86371064.88242364</v>
+      </c>
+      <c r="B26" t="n">
+        <v>12204845.78141508</v>
+      </c>
+      <c r="C26" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D26" t="n">
+        <v>36483821.3688428</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>48688667.15025788</v>
+      </c>
+      <c r="G26" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H26" t="n">
+        <v>24651641.5573359</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" t="n">
+        <v>7260733.901533453</v>
+      </c>
+      <c r="M26" t="n">
+        <v>86371064.88242364</v>
+      </c>
+      <c r="N26" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O26" t="n">
+        <v>0</v>
+      </c>
+      <c r="P26" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R26" t="n">
+        <v>0</v>
+      </c>
+      <c r="S26" t="n">
+        <v>0</v>
+      </c>
+      <c r="T26" t="n">
+        <v>0</v>
+      </c>
+      <c r="U26" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V26" t="n">
+        <v>6.976000070571899</v>
+      </c>
+      <c r="W26" t="n">
+        <v>86227475.51011334</v>
+      </c>
+      <c r="X26" t="n">
+        <v>86371064.88242364</v>
+      </c>
+      <c r="Y26" t="n">
+        <v>143589.3723102957</v>
+      </c>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD26" t="inlineStr">
+        <is>
+          <t>carbon_tax_50_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE26" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308182140_carbon_tax_50_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>76640249.08353671</v>
+      </c>
+      <c r="B27" t="n">
+        <v>12204845.78141508</v>
+      </c>
+      <c r="C27" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D27" t="n">
+        <v>36483821.3688428</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>48688667.15025788</v>
+      </c>
+      <c r="G27" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H27" t="n">
+        <v>7660091.856915521</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" t="n">
+        <v>14521467.80306691</v>
+      </c>
+      <c r="M27" t="n">
+        <v>76640249.08353671</v>
+      </c>
+      <c r="N27" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R27" t="n">
+        <v>0</v>
+      </c>
+      <c r="S27" t="n">
+        <v>0</v>
+      </c>
+      <c r="T27" t="n">
+        <v>0</v>
+      </c>
+      <c r="U27" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V27" t="n">
+        <v>7.562000036239624</v>
+      </c>
+      <c r="W27" t="n">
+        <v>76547740.66807944</v>
+      </c>
+      <c r="X27" t="n">
+        <v>76640249.08353671</v>
+      </c>
+      <c r="Y27" t="n">
+        <v>92508.41545727849</v>
+      </c>
+      <c r="Z27" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD27" t="inlineStr">
+        <is>
+          <t>carbon_tax_100_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE27" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308182507_carbon_tax_100_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>82304098.98367679</v>
+      </c>
+      <c r="B28" t="n">
+        <v>12204845.78141508</v>
+      </c>
+      <c r="C28" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D28" t="n">
+        <v>36483821.3688428</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>48688667.15025788</v>
+      </c>
+      <c r="G28" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H28" t="n">
+        <v>13323941.7570556</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" t="n">
+        <v>14521467.80306691</v>
+      </c>
+      <c r="M28" t="n">
+        <v>82304098.98367679</v>
+      </c>
+      <c r="N28" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R28" t="n">
+        <v>0</v>
+      </c>
+      <c r="S28" t="n">
+        <v>0</v>
+      </c>
+      <c r="T28" t="n">
+        <v>0</v>
+      </c>
+      <c r="U28" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V28" t="n">
+        <v>7.638999938964844</v>
+      </c>
+      <c r="W28" t="n">
+        <v>82211590.56821966</v>
+      </c>
+      <c r="X28" t="n">
+        <v>82304098.98367679</v>
+      </c>
+      <c r="Y28" t="n">
+        <v>92508.41545712948</v>
+      </c>
+      <c r="Z28" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD28" t="inlineStr">
+        <is>
+          <t>carbon_tax_100_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE28" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308182843_carbon_tax_100_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>87967948.88381693</v>
+      </c>
+      <c r="B29" t="n">
+        <v>12204845.78141508</v>
+      </c>
+      <c r="C29" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D29" t="n">
+        <v>36483821.3688428</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="n">
+        <v>48688667.15025788</v>
+      </c>
+      <c r="G29" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H29" t="n">
+        <v>18987791.65719574</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" t="n">
+        <v>14521467.80306691</v>
+      </c>
+      <c r="M29" t="n">
+        <v>87967948.88381693</v>
+      </c>
+      <c r="N29" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P29" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R29" t="n">
+        <v>0</v>
+      </c>
+      <c r="S29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T29" t="n">
+        <v>0</v>
+      </c>
+      <c r="U29" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V29" t="n">
+        <v>7.525000095367432</v>
+      </c>
+      <c r="W29" t="n">
+        <v>87875440.46835947</v>
+      </c>
+      <c r="X29" t="n">
+        <v>87967948.88381693</v>
+      </c>
+      <c r="Y29" t="n">
+        <v>92508.4154574573</v>
+      </c>
+      <c r="Z29" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD29" t="inlineStr">
+        <is>
+          <t>carbon_tax_100_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE29" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308183234_carbon_tax_100_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>93631798.78395709</v>
+      </c>
+      <c r="B30" t="n">
+        <v>12204845.78141508</v>
+      </c>
+      <c r="C30" t="n">
+        <v>5770022.273296408</v>
+      </c>
+      <c r="D30" t="n">
+        <v>36483821.3688428</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>48688667.15025788</v>
+      </c>
+      <c r="G30" t="n">
+        <v>5770022.273296408</v>
+      </c>
+      <c r="H30" t="n">
+        <v>24651641.5573359</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" t="n">
+        <v>14521467.80306691</v>
+      </c>
+      <c r="M30" t="n">
+        <v>93631798.78395709</v>
+      </c>
+      <c r="N30" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O30" t="n">
+        <v>0</v>
+      </c>
+      <c r="P30" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S30" t="n">
+        <v>0</v>
+      </c>
+      <c r="T30" t="n">
+        <v>0</v>
+      </c>
+      <c r="U30" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V30" t="n">
+        <v>6.767999887466431</v>
+      </c>
+      <c r="W30" t="n">
+        <v>93488209.41162935</v>
+      </c>
+      <c r="X30" t="n">
+        <v>93631798.78395709</v>
+      </c>
+      <c r="Y30" t="n">
+        <v>143589.372327745</v>
+      </c>
+      <c r="Z30" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA30" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD30" t="inlineStr">
+        <is>
+          <t>carbon_tax_100_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE30" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308183639_carbon_tax_100_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>83900982.98507082</v>
+      </c>
+      <c r="B31" t="n">
+        <v>12204845.78141508</v>
+      </c>
+      <c r="C31" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D31" t="n">
+        <v>36483821.3688428</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>48688667.15025788</v>
+      </c>
+      <c r="G31" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H31" t="n">
+        <v>7660091.856915521</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" t="n">
+        <v>21782201.70460102</v>
+      </c>
+      <c r="M31" t="n">
+        <v>83900982.98507082</v>
+      </c>
+      <c r="N31" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O31" t="n">
+        <v>0</v>
+      </c>
+      <c r="P31" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R31" t="n">
+        <v>0</v>
+      </c>
+      <c r="S31" t="n">
+        <v>0</v>
+      </c>
+      <c r="T31" t="n">
+        <v>0</v>
+      </c>
+      <c r="U31" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V31" t="n">
+        <v>7.427999973297119</v>
+      </c>
+      <c r="W31" t="n">
+        <v>83808474.5696134</v>
+      </c>
+      <c r="X31" t="n">
+        <v>83900982.98507082</v>
+      </c>
+      <c r="Y31" t="n">
+        <v>92508.4154574275</v>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD31" t="inlineStr">
+        <is>
+          <t>carbon_tax_150_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE31" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308183925_carbon_tax_150_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>89564832.8852109</v>
+      </c>
+      <c r="B32" t="n">
+        <v>12204845.78141508</v>
+      </c>
+      <c r="C32" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D32" t="n">
+        <v>36483821.3688428</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="n">
+        <v>48688667.15025788</v>
+      </c>
+      <c r="G32" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H32" t="n">
+        <v>13323941.7570556</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" t="n">
+        <v>21782201.70460102</v>
+      </c>
+      <c r="M32" t="n">
+        <v>89564832.8852109</v>
+      </c>
+      <c r="N32" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O32" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R32" t="n">
+        <v>0</v>
+      </c>
+      <c r="S32" t="n">
+        <v>0</v>
+      </c>
+      <c r="T32" t="n">
+        <v>0</v>
+      </c>
+      <c r="U32" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V32" t="n">
+        <v>7.723999977111816</v>
+      </c>
+      <c r="W32" t="n">
+        <v>89472324.46975398</v>
+      </c>
+      <c r="X32" t="n">
+        <v>89564832.8852109</v>
+      </c>
+      <c r="Y32" t="n">
+        <v>92508.41545692086</v>
+      </c>
+      <c r="Z32" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD32" t="inlineStr">
+        <is>
+          <t>carbon_tax_150_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE32" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308184345_carbon_tax_150_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>95228682.78535104</v>
+      </c>
+      <c r="B33" t="n">
+        <v>12204845.78141508</v>
+      </c>
+      <c r="C33" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D33" t="n">
+        <v>36483821.3688428</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="n">
+        <v>48688667.15025788</v>
+      </c>
+      <c r="G33" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H33" t="n">
+        <v>18987791.65719574</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" t="n">
+        <v>21782201.70460102</v>
+      </c>
+      <c r="M33" t="n">
+        <v>95228682.78535104</v>
+      </c>
+      <c r="N33" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O33" t="n">
+        <v>0</v>
+      </c>
+      <c r="P33" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R33" t="n">
+        <v>0</v>
+      </c>
+      <c r="S33" t="n">
+        <v>0</v>
+      </c>
+      <c r="T33" t="n">
+        <v>0</v>
+      </c>
+      <c r="U33" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V33" t="n">
+        <v>8.078000068664551</v>
+      </c>
+      <c r="W33" t="n">
+        <v>95136174.36989495</v>
+      </c>
+      <c r="X33" t="n">
+        <v>95228682.78535104</v>
+      </c>
+      <c r="Y33" t="n">
+        <v>92508.4154560864</v>
+      </c>
+      <c r="Z33" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD33" t="inlineStr">
+        <is>
+          <t>carbon_tax_150_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE33" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308184630_carbon_tax_150_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>100892532.6854912</v>
+      </c>
+      <c r="B34" t="n">
+        <v>12204845.78141508</v>
+      </c>
+      <c r="C34" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D34" t="n">
+        <v>36483821.3688428</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="n">
+        <v>48688667.15025788</v>
+      </c>
+      <c r="G34" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H34" t="n">
+        <v>24651641.5573359</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" t="n">
+        <v>21782201.70460102</v>
+      </c>
+      <c r="M34" t="n">
+        <v>100892532.6854912</v>
+      </c>
+      <c r="N34" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O34" t="n">
+        <v>0</v>
+      </c>
+      <c r="P34" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R34" t="n">
+        <v>0</v>
+      </c>
+      <c r="S34" t="n">
+        <v>0</v>
+      </c>
+      <c r="T34" t="n">
+        <v>0</v>
+      </c>
+      <c r="U34" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V34" t="n">
+        <v>8.915999889373779</v>
+      </c>
+      <c r="W34" t="n">
+        <v>100800024.2700393</v>
+      </c>
+      <c r="X34" t="n">
+        <v>100892532.6854912</v>
+      </c>
+      <c r="Y34" t="n">
+        <v>92508.41545194387</v>
+      </c>
+      <c r="Z34" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA34" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD34" t="inlineStr">
+        <is>
+          <t>carbon_tax_150_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE34" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308185114_carbon_tax_150_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>87221015.94520186</v>
+      </c>
+      <c r="B35" t="n">
+        <v>19553428.22612901</v>
+      </c>
+      <c r="C35" t="n">
+        <v>6740380.891781891</v>
+      </c>
+      <c r="D35" t="n">
+        <v>50831547.95827343</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>70384976.18440245</v>
+      </c>
+      <c r="G35" t="n">
+        <v>6740380.891781891</v>
+      </c>
+      <c r="H35" t="n">
+        <v>8643512.088710817</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" t="n">
+        <v>1452146.780306702</v>
+      </c>
+      <c r="M35" t="n">
+        <v>87221015.94520186</v>
+      </c>
+      <c r="N35" t="n">
+        <v>7268.969672063526</v>
+      </c>
+      <c r="O35" t="n">
+        <v>0</v>
+      </c>
+      <c r="P35" t="n">
+        <v>7268.969672063526</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>7260.733901533531</v>
+      </c>
+      <c r="R35" t="n">
+        <v>0</v>
+      </c>
+      <c r="S35" t="n">
+        <v>0</v>
+      </c>
+      <c r="T35" t="n">
+        <v>0</v>
+      </c>
+      <c r="U35" t="n">
+        <v>8.235770529824357</v>
+      </c>
+      <c r="V35" t="n">
+        <v>11.29399991035461</v>
+      </c>
+      <c r="W35" t="n">
+        <v>87221015.94517553</v>
+      </c>
+      <c r="X35" t="n">
+        <v>87221015.94520186</v>
+      </c>
+      <c r="Y35" t="n">
+        <v>2.633035182952881e-05</v>
+      </c>
+      <c r="Z35" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD35" t="inlineStr">
+        <is>
+          <t>carbon_tax_200_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE35" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308185401_carbon_tax_200_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>93868286.07713728</v>
+      </c>
+      <c r="B36" t="n">
+        <v>19553428.22612901</v>
+      </c>
+      <c r="C36" t="n">
+        <v>6740380.891781891</v>
+      </c>
+      <c r="D36" t="n">
+        <v>50831547.95827343</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="n">
+        <v>70384976.18440245</v>
+      </c>
+      <c r="G36" t="n">
+        <v>6740380.891781891</v>
+      </c>
+      <c r="H36" t="n">
+        <v>15290782.22064623</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" t="n">
+        <v>1452146.780306702</v>
+      </c>
+      <c r="M36" t="n">
+        <v>93868286.07713728</v>
+      </c>
+      <c r="N36" t="n">
+        <v>7268.969672063526</v>
+      </c>
+      <c r="O36" t="n">
+        <v>0</v>
+      </c>
+      <c r="P36" t="n">
+        <v>7268.969672063526</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>7260.733901533531</v>
+      </c>
+      <c r="R36" t="n">
+        <v>0</v>
+      </c>
+      <c r="S36" t="n">
+        <v>0</v>
+      </c>
+      <c r="T36" t="n">
+        <v>0</v>
+      </c>
+      <c r="U36" t="n">
+        <v>8.235770529824357</v>
+      </c>
+      <c r="V36" t="n">
+        <v>11.28999996185303</v>
+      </c>
+      <c r="W36" t="n">
+        <v>93868286.0771116</v>
+      </c>
+      <c r="X36" t="n">
+        <v>93868286.07713728</v>
+      </c>
+      <c r="Y36" t="n">
+        <v>2.567470073699951e-05</v>
+      </c>
+      <c r="Z36" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA36" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC36" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD36" t="inlineStr">
+        <is>
+          <t>carbon_tax_200_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE36" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308185914_carbon_tax_200_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>102489416.6868838</v>
+      </c>
+      <c r="B37" t="n">
+        <v>12204845.78141508</v>
+      </c>
+      <c r="C37" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D37" t="n">
+        <v>36483821.3688428</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="n">
+        <v>48688667.15025788</v>
+      </c>
+      <c r="G37" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H37" t="n">
+        <v>18987791.65719574</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" t="n">
+        <v>29042935.60613381</v>
+      </c>
+      <c r="M37" t="n">
+        <v>102489416.6868838</v>
+      </c>
+      <c r="N37" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O37" t="n">
+        <v>0</v>
+      </c>
+      <c r="P37" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R37" t="n">
+        <v>0</v>
+      </c>
+      <c r="S37" t="n">
+        <v>0</v>
+      </c>
+      <c r="T37" t="n">
+        <v>0</v>
+      </c>
+      <c r="U37" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V37" t="n">
+        <v>11.62599992752075</v>
+      </c>
+      <c r="W37" t="n">
+        <v>100478856.6206367</v>
+      </c>
+      <c r="X37" t="n">
+        <v>102489416.6868838</v>
+      </c>
+      <c r="Y37" t="n">
+        <v>2010560.06624718</v>
+      </c>
+      <c r="Z37" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA37" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC37" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD37" t="inlineStr">
+        <is>
+          <t>carbon_tax_200_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE37" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308190204_carbon_tax_200_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>108153266.587024</v>
+      </c>
+      <c r="B38" t="n">
+        <v>12204845.78141508</v>
+      </c>
+      <c r="C38" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D38" t="n">
+        <v>36483821.3688428</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" t="n">
+        <v>48688667.15025788</v>
+      </c>
+      <c r="G38" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H38" t="n">
+        <v>24651641.5573359</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" t="n">
+        <v>0</v>
+      </c>
+      <c r="K38" t="n">
+        <v>0</v>
+      </c>
+      <c r="L38" t="n">
+        <v>29042935.60613381</v>
+      </c>
+      <c r="M38" t="n">
+        <v>108153266.587024</v>
+      </c>
+      <c r="N38" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O38" t="n">
+        <v>0</v>
+      </c>
+      <c r="P38" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R38" t="n">
+        <v>0</v>
+      </c>
+      <c r="S38" t="n">
+        <v>0</v>
+      </c>
+      <c r="T38" t="n">
+        <v>0</v>
+      </c>
+      <c r="U38" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V38" t="n">
+        <v>10.11600017547607</v>
+      </c>
+      <c r="W38" t="n">
+        <v>106867380.5452164</v>
+      </c>
+      <c r="X38" t="n">
+        <v>108153266.587024</v>
+      </c>
+      <c r="Y38" t="n">
+        <v>1285886.041807592</v>
+      </c>
+      <c r="Z38" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA38" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC38" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD38" t="inlineStr">
+        <is>
+          <t>carbon_tax_200_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE38" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308190453_carbon_tax_200_el_price_200</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
results cement tech selection updated
</commit_message>
<xml_diff>
--- a/dataCaseStudy_Cement/raw_results/tech_selection/Summary.xlsx
+++ b/dataCaseStudy_Cement/raw_results/tech_selection/Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE38"/>
+  <dimension ref="A1:AE54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4393,6 +4393,1654 @@
       <c r="AE38" t="inlineStr">
         <is>
           <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308190453_carbon_tax_200_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>69379515.18200339</v>
+      </c>
+      <c r="B39" t="n">
+        <v>12204845.78141507</v>
+      </c>
+      <c r="C39" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D39" t="n">
+        <v>36483821.36884278</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" t="n">
+        <v>48688667.15025785</v>
+      </c>
+      <c r="G39" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H39" t="n">
+        <v>7660091.856915681</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0</v>
+      </c>
+      <c r="L39" t="n">
+        <v>7260733.901533453</v>
+      </c>
+      <c r="M39" t="n">
+        <v>69379515.18200339</v>
+      </c>
+      <c r="N39" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O39" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R39" t="n">
+        <v>0</v>
+      </c>
+      <c r="S39" t="n">
+        <v>0</v>
+      </c>
+      <c r="T39" t="n">
+        <v>0</v>
+      </c>
+      <c r="U39" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V39" t="n">
+        <v>2.718999862670898</v>
+      </c>
+      <c r="W39" t="n">
+        <v>69379515.18200339</v>
+      </c>
+      <c r="X39" t="n">
+        <v>69379515.18200339</v>
+      </c>
+      <c r="Y39" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z39" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA39" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD39" t="inlineStr">
+        <is>
+          <t>carbon_tax_50_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE39" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308221544_carbon_tax_50_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>75043365.08214357</v>
+      </c>
+      <c r="B40" t="n">
+        <v>12204845.78141507</v>
+      </c>
+      <c r="C40" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D40" t="n">
+        <v>36483821.36884278</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" t="n">
+        <v>48688667.15025785</v>
+      </c>
+      <c r="G40" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H40" t="n">
+        <v>13323941.75705586</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0</v>
+      </c>
+      <c r="J40" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" t="n">
+        <v>0</v>
+      </c>
+      <c r="L40" t="n">
+        <v>7260733.901533453</v>
+      </c>
+      <c r="M40" t="n">
+        <v>75043365.08214357</v>
+      </c>
+      <c r="N40" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O40" t="n">
+        <v>0</v>
+      </c>
+      <c r="P40" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R40" t="n">
+        <v>0</v>
+      </c>
+      <c r="S40" t="n">
+        <v>0</v>
+      </c>
+      <c r="T40" t="n">
+        <v>0</v>
+      </c>
+      <c r="U40" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V40" t="n">
+        <v>2.355000019073486</v>
+      </c>
+      <c r="W40" t="n">
+        <v>75043365.0821397</v>
+      </c>
+      <c r="X40" t="n">
+        <v>75043365.08214357</v>
+      </c>
+      <c r="Y40" t="n">
+        <v>3.874301910400391e-06</v>
+      </c>
+      <c r="Z40" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA40" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC40" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD40" t="inlineStr">
+        <is>
+          <t>carbon_tax_50_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE40" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308221759_carbon_tax_50_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>80707214.98228374</v>
+      </c>
+      <c r="B41" t="n">
+        <v>12204845.78141507</v>
+      </c>
+      <c r="C41" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D41" t="n">
+        <v>36483821.36884278</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" t="n">
+        <v>48688667.15025785</v>
+      </c>
+      <c r="G41" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H41" t="n">
+        <v>18987791.65719603</v>
+      </c>
+      <c r="I41" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" t="n">
+        <v>0</v>
+      </c>
+      <c r="L41" t="n">
+        <v>7260733.901533453</v>
+      </c>
+      <c r="M41" t="n">
+        <v>80707214.98228374</v>
+      </c>
+      <c r="N41" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O41" t="n">
+        <v>0</v>
+      </c>
+      <c r="P41" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R41" t="n">
+        <v>0</v>
+      </c>
+      <c r="S41" t="n">
+        <v>0</v>
+      </c>
+      <c r="T41" t="n">
+        <v>0</v>
+      </c>
+      <c r="U41" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V41" t="n">
+        <v>2.333999872207642</v>
+      </c>
+      <c r="W41" t="n">
+        <v>80707214.98227409</v>
+      </c>
+      <c r="X41" t="n">
+        <v>80707214.98228374</v>
+      </c>
+      <c r="Y41" t="n">
+        <v>9.655952453613281e-06</v>
+      </c>
+      <c r="Z41" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA41" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC41" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD41" t="inlineStr">
+        <is>
+          <t>carbon_tax_50_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE41" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308222019_carbon_tax_50_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>86371064.88242392</v>
+      </c>
+      <c r="B42" t="n">
+        <v>12204845.78141507</v>
+      </c>
+      <c r="C42" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D42" t="n">
+        <v>36483821.36884278</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" t="n">
+        <v>48688667.15025785</v>
+      </c>
+      <c r="G42" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H42" t="n">
+        <v>24651641.55733621</v>
+      </c>
+      <c r="I42" t="n">
+        <v>0</v>
+      </c>
+      <c r="J42" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" t="n">
+        <v>0</v>
+      </c>
+      <c r="L42" t="n">
+        <v>7260733.901533453</v>
+      </c>
+      <c r="M42" t="n">
+        <v>86371064.88242392</v>
+      </c>
+      <c r="N42" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O42" t="n">
+        <v>0</v>
+      </c>
+      <c r="P42" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R42" t="n">
+        <v>0</v>
+      </c>
+      <c r="S42" t="n">
+        <v>0</v>
+      </c>
+      <c r="T42" t="n">
+        <v>0</v>
+      </c>
+      <c r="U42" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V42" t="n">
+        <v>2.297999858856201</v>
+      </c>
+      <c r="W42" t="n">
+        <v>86371064.88240911</v>
+      </c>
+      <c r="X42" t="n">
+        <v>86371064.88242392</v>
+      </c>
+      <c r="Y42" t="n">
+        <v>1.481175422668457e-05</v>
+      </c>
+      <c r="Z42" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA42" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC42" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD42" t="inlineStr">
+        <is>
+          <t>carbon_tax_50_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE42" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308222241_carbon_tax_50_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>76640249.08353685</v>
+      </c>
+      <c r="B43" t="n">
+        <v>12204845.78141507</v>
+      </c>
+      <c r="C43" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D43" t="n">
+        <v>36483821.36884278</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" t="n">
+        <v>48688667.15025785</v>
+      </c>
+      <c r="G43" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H43" t="n">
+        <v>7660091.856915681</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" t="n">
+        <v>0</v>
+      </c>
+      <c r="K43" t="n">
+        <v>0</v>
+      </c>
+      <c r="L43" t="n">
+        <v>14521467.80306691</v>
+      </c>
+      <c r="M43" t="n">
+        <v>76640249.08353685</v>
+      </c>
+      <c r="N43" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O43" t="n">
+        <v>0</v>
+      </c>
+      <c r="P43" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R43" t="n">
+        <v>0</v>
+      </c>
+      <c r="S43" t="n">
+        <v>0</v>
+      </c>
+      <c r="T43" t="n">
+        <v>0</v>
+      </c>
+      <c r="U43" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V43" t="n">
+        <v>2.276000022888184</v>
+      </c>
+      <c r="W43" t="n">
+        <v>76640249.08353685</v>
+      </c>
+      <c r="X43" t="n">
+        <v>76640249.08353685</v>
+      </c>
+      <c r="Y43" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z43" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA43" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC43" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD43" t="inlineStr">
+        <is>
+          <t>carbon_tax_100_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE43" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308222455_carbon_tax_100_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>82304098.98367703</v>
+      </c>
+      <c r="B44" t="n">
+        <v>12204845.78141507</v>
+      </c>
+      <c r="C44" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D44" t="n">
+        <v>36483821.36884278</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" t="n">
+        <v>48688667.15025785</v>
+      </c>
+      <c r="G44" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H44" t="n">
+        <v>13323941.75705586</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" t="n">
+        <v>0</v>
+      </c>
+      <c r="L44" t="n">
+        <v>14521467.80306691</v>
+      </c>
+      <c r="M44" t="n">
+        <v>82304098.98367703</v>
+      </c>
+      <c r="N44" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O44" t="n">
+        <v>0</v>
+      </c>
+      <c r="P44" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R44" t="n">
+        <v>0</v>
+      </c>
+      <c r="S44" t="n">
+        <v>0</v>
+      </c>
+      <c r="T44" t="n">
+        <v>0</v>
+      </c>
+      <c r="U44" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V44" t="n">
+        <v>2.236999988555908</v>
+      </c>
+      <c r="W44" t="n">
+        <v>82304098.98367703</v>
+      </c>
+      <c r="X44" t="n">
+        <v>82304098.98367703</v>
+      </c>
+      <c r="Y44" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z44" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA44" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC44" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD44" t="inlineStr">
+        <is>
+          <t>carbon_tax_100_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE44" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308222712_carbon_tax_100_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>87967948.8838172</v>
+      </c>
+      <c r="B45" t="n">
+        <v>12204845.78141507</v>
+      </c>
+      <c r="C45" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D45" t="n">
+        <v>36483821.36884278</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" t="n">
+        <v>48688667.15025785</v>
+      </c>
+      <c r="G45" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H45" t="n">
+        <v>18987791.65719603</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" t="n">
+        <v>14521467.80306691</v>
+      </c>
+      <c r="M45" t="n">
+        <v>87967948.8838172</v>
+      </c>
+      <c r="N45" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O45" t="n">
+        <v>0</v>
+      </c>
+      <c r="P45" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R45" t="n">
+        <v>0</v>
+      </c>
+      <c r="S45" t="n">
+        <v>0</v>
+      </c>
+      <c r="T45" t="n">
+        <v>0</v>
+      </c>
+      <c r="U45" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V45" t="n">
+        <v>2.319000005722046</v>
+      </c>
+      <c r="W45" t="n">
+        <v>87967948.88381673</v>
+      </c>
+      <c r="X45" t="n">
+        <v>87967948.8838172</v>
+      </c>
+      <c r="Y45" t="n">
+        <v>4.619359970092773e-07</v>
+      </c>
+      <c r="Z45" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA45" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC45" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD45" t="inlineStr">
+        <is>
+          <t>carbon_tax_100_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE45" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308222936_carbon_tax_100_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>93631798.78395738</v>
+      </c>
+      <c r="B46" t="n">
+        <v>12204845.78141507</v>
+      </c>
+      <c r="C46" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D46" t="n">
+        <v>36483821.36884278</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" t="n">
+        <v>48688667.15025785</v>
+      </c>
+      <c r="G46" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H46" t="n">
+        <v>24651641.55733621</v>
+      </c>
+      <c r="I46" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" t="n">
+        <v>0</v>
+      </c>
+      <c r="L46" t="n">
+        <v>14521467.80306691</v>
+      </c>
+      <c r="M46" t="n">
+        <v>93631798.78395738</v>
+      </c>
+      <c r="N46" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O46" t="n">
+        <v>0</v>
+      </c>
+      <c r="P46" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R46" t="n">
+        <v>0</v>
+      </c>
+      <c r="S46" t="n">
+        <v>0</v>
+      </c>
+      <c r="T46" t="n">
+        <v>0</v>
+      </c>
+      <c r="U46" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V46" t="n">
+        <v>2.315000057220459</v>
+      </c>
+      <c r="W46" t="n">
+        <v>93631798.7839521</v>
+      </c>
+      <c r="X46" t="n">
+        <v>93631798.78395738</v>
+      </c>
+      <c r="Y46" t="n">
+        <v>5.27501106262207e-06</v>
+      </c>
+      <c r="Z46" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA46" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC46" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD46" t="inlineStr">
+        <is>
+          <t>carbon_tax_100_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE46" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308223210_carbon_tax_100_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>83900982.98507096</v>
+      </c>
+      <c r="B47" t="n">
+        <v>12204845.78141507</v>
+      </c>
+      <c r="C47" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D47" t="n">
+        <v>36483821.36884278</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" t="n">
+        <v>48688667.15025785</v>
+      </c>
+      <c r="G47" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H47" t="n">
+        <v>7660091.856915681</v>
+      </c>
+      <c r="I47" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" t="n">
+        <v>0</v>
+      </c>
+      <c r="K47" t="n">
+        <v>0</v>
+      </c>
+      <c r="L47" t="n">
+        <v>21782201.70460102</v>
+      </c>
+      <c r="M47" t="n">
+        <v>83900982.98507096</v>
+      </c>
+      <c r="N47" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O47" t="n">
+        <v>0</v>
+      </c>
+      <c r="P47" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R47" t="n">
+        <v>0</v>
+      </c>
+      <c r="S47" t="n">
+        <v>0</v>
+      </c>
+      <c r="T47" t="n">
+        <v>0</v>
+      </c>
+      <c r="U47" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V47" t="n">
+        <v>2.300999879837036</v>
+      </c>
+      <c r="W47" t="n">
+        <v>83900982.98507096</v>
+      </c>
+      <c r="X47" t="n">
+        <v>83900982.98507096</v>
+      </c>
+      <c r="Y47" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z47" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA47" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC47" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD47" t="inlineStr">
+        <is>
+          <t>carbon_tax_150_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE47" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308223401_carbon_tax_150_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>89564832.88521114</v>
+      </c>
+      <c r="B48" t="n">
+        <v>12204845.78141507</v>
+      </c>
+      <c r="C48" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D48" t="n">
+        <v>36483821.36884278</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" t="n">
+        <v>48688667.15025785</v>
+      </c>
+      <c r="G48" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H48" t="n">
+        <v>13323941.75705586</v>
+      </c>
+      <c r="I48" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" t="n">
+        <v>0</v>
+      </c>
+      <c r="K48" t="n">
+        <v>0</v>
+      </c>
+      <c r="L48" t="n">
+        <v>21782201.70460102</v>
+      </c>
+      <c r="M48" t="n">
+        <v>89564832.88521114</v>
+      </c>
+      <c r="N48" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O48" t="n">
+        <v>0</v>
+      </c>
+      <c r="P48" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R48" t="n">
+        <v>0</v>
+      </c>
+      <c r="S48" t="n">
+        <v>0</v>
+      </c>
+      <c r="T48" t="n">
+        <v>0</v>
+      </c>
+      <c r="U48" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V48" t="n">
+        <v>2.289999961853027</v>
+      </c>
+      <c r="W48" t="n">
+        <v>89564832.88521114</v>
+      </c>
+      <c r="X48" t="n">
+        <v>89564832.88521114</v>
+      </c>
+      <c r="Y48" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z48" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA48" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC48" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD48" t="inlineStr">
+        <is>
+          <t>carbon_tax_150_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE48" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308223642_carbon_tax_150_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>95228682.78535131</v>
+      </c>
+      <c r="B49" t="n">
+        <v>12204845.78141507</v>
+      </c>
+      <c r="C49" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D49" t="n">
+        <v>36483821.36884278</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" t="n">
+        <v>48688667.15025785</v>
+      </c>
+      <c r="G49" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H49" t="n">
+        <v>18987791.65719603</v>
+      </c>
+      <c r="I49" t="n">
+        <v>0</v>
+      </c>
+      <c r="J49" t="n">
+        <v>0</v>
+      </c>
+      <c r="K49" t="n">
+        <v>0</v>
+      </c>
+      <c r="L49" t="n">
+        <v>21782201.70460102</v>
+      </c>
+      <c r="M49" t="n">
+        <v>95228682.78535131</v>
+      </c>
+      <c r="N49" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O49" t="n">
+        <v>0</v>
+      </c>
+      <c r="P49" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R49" t="n">
+        <v>0</v>
+      </c>
+      <c r="S49" t="n">
+        <v>0</v>
+      </c>
+      <c r="T49" t="n">
+        <v>0</v>
+      </c>
+      <c r="U49" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V49" t="n">
+        <v>2.032999992370605</v>
+      </c>
+      <c r="W49" t="n">
+        <v>95228682.78535131</v>
+      </c>
+      <c r="X49" t="n">
+        <v>95228682.78535131</v>
+      </c>
+      <c r="Y49" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z49" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA49" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC49" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD49" t="inlineStr">
+        <is>
+          <t>carbon_tax_150_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE49" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308223834_carbon_tax_150_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>100892532.6854915</v>
+      </c>
+      <c r="B50" t="n">
+        <v>12204845.78141507</v>
+      </c>
+      <c r="C50" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="D50" t="n">
+        <v>36483821.36884278</v>
+      </c>
+      <c r="E50" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" t="n">
+        <v>48688667.15025785</v>
+      </c>
+      <c r="G50" t="n">
+        <v>5770022.273296411</v>
+      </c>
+      <c r="H50" t="n">
+        <v>24651641.55733621</v>
+      </c>
+      <c r="I50" t="n">
+        <v>0</v>
+      </c>
+      <c r="J50" t="n">
+        <v>0</v>
+      </c>
+      <c r="K50" t="n">
+        <v>0</v>
+      </c>
+      <c r="L50" t="n">
+        <v>21782201.70460102</v>
+      </c>
+      <c r="M50" t="n">
+        <v>100892532.6854915</v>
+      </c>
+      <c r="N50" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="O50" t="n">
+        <v>0</v>
+      </c>
+      <c r="P50" t="n">
+        <v>145221.189376899</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>145214.6780306711</v>
+      </c>
+      <c r="R50" t="n">
+        <v>0</v>
+      </c>
+      <c r="S50" t="n">
+        <v>0</v>
+      </c>
+      <c r="T50" t="n">
+        <v>0</v>
+      </c>
+      <c r="U50" t="n">
+        <v>6.511346228210139</v>
+      </c>
+      <c r="V50" t="n">
+        <v>1.993000030517578</v>
+      </c>
+      <c r="W50" t="n">
+        <v>100892532.6854915</v>
+      </c>
+      <c r="X50" t="n">
+        <v>100892532.6854915</v>
+      </c>
+      <c r="Y50" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z50" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA50" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC50" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD50" t="inlineStr">
+        <is>
+          <t>carbon_tax_150_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE50" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308224123_carbon_tax_150_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>87221015.94520204</v>
+      </c>
+      <c r="B51" t="n">
+        <v>19553428.22612903</v>
+      </c>
+      <c r="C51" t="n">
+        <v>6740380.891781893</v>
+      </c>
+      <c r="D51" t="n">
+        <v>50831547.95827347</v>
+      </c>
+      <c r="E51" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" t="n">
+        <v>70384976.1844025</v>
+      </c>
+      <c r="G51" t="n">
+        <v>6740380.891781893</v>
+      </c>
+      <c r="H51" t="n">
+        <v>8643512.088711005</v>
+      </c>
+      <c r="I51" t="n">
+        <v>0</v>
+      </c>
+      <c r="J51" t="n">
+        <v>0</v>
+      </c>
+      <c r="K51" t="n">
+        <v>0</v>
+      </c>
+      <c r="L51" t="n">
+        <v>1452146.780306642</v>
+      </c>
+      <c r="M51" t="n">
+        <v>87221015.94520204</v>
+      </c>
+      <c r="N51" t="n">
+        <v>7268.969672062963</v>
+      </c>
+      <c r="O51" t="n">
+        <v>0</v>
+      </c>
+      <c r="P51" t="n">
+        <v>7268.969672062963</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>7260.733901533139</v>
+      </c>
+      <c r="R51" t="n">
+        <v>0</v>
+      </c>
+      <c r="S51" t="n">
+        <v>0</v>
+      </c>
+      <c r="T51" t="n">
+        <v>0</v>
+      </c>
+      <c r="U51" t="n">
+        <v>8.235770529824363</v>
+      </c>
+      <c r="V51" t="n">
+        <v>2.305999994277954</v>
+      </c>
+      <c r="W51" t="n">
+        <v>87221015.94520204</v>
+      </c>
+      <c r="X51" t="n">
+        <v>87221015.94520204</v>
+      </c>
+      <c r="Y51" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z51" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA51" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC51" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD51" t="inlineStr">
+        <is>
+          <t>carbon_tax_200_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE51" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308224312_carbon_tax_200_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>93868286.07713753</v>
+      </c>
+      <c r="B52" t="n">
+        <v>19553428.22612903</v>
+      </c>
+      <c r="C52" t="n">
+        <v>6740380.891781893</v>
+      </c>
+      <c r="D52" t="n">
+        <v>50831547.95827347</v>
+      </c>
+      <c r="E52" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" t="n">
+        <v>70384976.1844025</v>
+      </c>
+      <c r="G52" t="n">
+        <v>6740380.891781893</v>
+      </c>
+      <c r="H52" t="n">
+        <v>15290782.22064651</v>
+      </c>
+      <c r="I52" t="n">
+        <v>0</v>
+      </c>
+      <c r="J52" t="n">
+        <v>0</v>
+      </c>
+      <c r="K52" t="n">
+        <v>0</v>
+      </c>
+      <c r="L52" t="n">
+        <v>1452146.780306642</v>
+      </c>
+      <c r="M52" t="n">
+        <v>93868286.07713753</v>
+      </c>
+      <c r="N52" t="n">
+        <v>7268.969672062963</v>
+      </c>
+      <c r="O52" t="n">
+        <v>0</v>
+      </c>
+      <c r="P52" t="n">
+        <v>7268.969672062963</v>
+      </c>
+      <c r="Q52" t="n">
+        <v>7260.733901533139</v>
+      </c>
+      <c r="R52" t="n">
+        <v>0</v>
+      </c>
+      <c r="S52" t="n">
+        <v>0</v>
+      </c>
+      <c r="T52" t="n">
+        <v>0</v>
+      </c>
+      <c r="U52" t="n">
+        <v>8.235770529824363</v>
+      </c>
+      <c r="V52" t="n">
+        <v>2.163000106811523</v>
+      </c>
+      <c r="W52" t="n">
+        <v>93868286.07713753</v>
+      </c>
+      <c r="X52" t="n">
+        <v>93868286.07713753</v>
+      </c>
+      <c r="Y52" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z52" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA52" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB52" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC52" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD52" t="inlineStr">
+        <is>
+          <t>carbon_tax_200_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE52" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308224614_carbon_tax_200_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>100515556.2090731</v>
+      </c>
+      <c r="B53" t="n">
+        <v>19553428.22612903</v>
+      </c>
+      <c r="C53" t="n">
+        <v>6740380.891781893</v>
+      </c>
+      <c r="D53" t="n">
+        <v>50831547.95827347</v>
+      </c>
+      <c r="E53" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" t="n">
+        <v>70384976.1844025</v>
+      </c>
+      <c r="G53" t="n">
+        <v>6740380.891781893</v>
+      </c>
+      <c r="H53" t="n">
+        <v>21938052.35258202</v>
+      </c>
+      <c r="I53" t="n">
+        <v>0</v>
+      </c>
+      <c r="J53" t="n">
+        <v>0</v>
+      </c>
+      <c r="K53" t="n">
+        <v>0</v>
+      </c>
+      <c r="L53" t="n">
+        <v>1452146.780306642</v>
+      </c>
+      <c r="M53" t="n">
+        <v>100515556.2090731</v>
+      </c>
+      <c r="N53" t="n">
+        <v>7268.969672062963</v>
+      </c>
+      <c r="O53" t="n">
+        <v>0</v>
+      </c>
+      <c r="P53" t="n">
+        <v>7268.969672062963</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>7260.733901533139</v>
+      </c>
+      <c r="R53" t="n">
+        <v>0</v>
+      </c>
+      <c r="S53" t="n">
+        <v>0</v>
+      </c>
+      <c r="T53" t="n">
+        <v>0</v>
+      </c>
+      <c r="U53" t="n">
+        <v>8.235770529824363</v>
+      </c>
+      <c r="V53" t="n">
+        <v>2.246999979019165</v>
+      </c>
+      <c r="W53" t="n">
+        <v>100515556.2090731</v>
+      </c>
+      <c r="X53" t="n">
+        <v>100515556.2090731</v>
+      </c>
+      <c r="Y53" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z53" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA53" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC53" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD53" t="inlineStr">
+        <is>
+          <t>carbon_tax_200_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE53" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308224804_carbon_tax_200_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>107162826.3410085</v>
+      </c>
+      <c r="B54" t="n">
+        <v>19553428.22612903</v>
+      </c>
+      <c r="C54" t="n">
+        <v>6740380.891781893</v>
+      </c>
+      <c r="D54" t="n">
+        <v>50831547.95827347</v>
+      </c>
+      <c r="E54" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" t="n">
+        <v>70384976.1844025</v>
+      </c>
+      <c r="G54" t="n">
+        <v>6740380.891781893</v>
+      </c>
+      <c r="H54" t="n">
+        <v>28585322.48451751</v>
+      </c>
+      <c r="I54" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" t="n">
+        <v>0</v>
+      </c>
+      <c r="K54" t="n">
+        <v>0</v>
+      </c>
+      <c r="L54" t="n">
+        <v>1452146.780306642</v>
+      </c>
+      <c r="M54" t="n">
+        <v>107162826.3410085</v>
+      </c>
+      <c r="N54" t="n">
+        <v>7268.969672062963</v>
+      </c>
+      <c r="O54" t="n">
+        <v>0</v>
+      </c>
+      <c r="P54" t="n">
+        <v>7268.969672062963</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>7260.733901533139</v>
+      </c>
+      <c r="R54" t="n">
+        <v>0</v>
+      </c>
+      <c r="S54" t="n">
+        <v>0</v>
+      </c>
+      <c r="T54" t="n">
+        <v>0</v>
+      </c>
+      <c r="U54" t="n">
+        <v>8.235770529824363</v>
+      </c>
+      <c r="V54" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="W54" t="n">
+        <v>107162826.3410085</v>
+      </c>
+      <c r="X54" t="n">
+        <v>107162826.3410085</v>
+      </c>
+      <c r="Y54" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z54" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA54" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD54" t="inlineStr">
+        <is>
+          <t>carbon_tax_200_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE54" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260308224953_carbon_tax_200_el_price_200</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Results tech selection cement 2.0
</commit_message>
<xml_diff>
--- a/dataCaseStudy_Cement/raw_results/tech_selection/Summary.xlsx
+++ b/dataCaseStudy_Cement/raw_results/tech_selection/Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE168"/>
+  <dimension ref="A1:AE193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17783,6 +17783,2581 @@
       <c r="AE168" t="inlineStr">
         <is>
           <t>dataCaseStudy_Cement\raw_results\tech_selection\20260403224914_carbon_tax_300_el_price_250</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="n">
+        <v>50918225.93967282</v>
+      </c>
+      <c r="B169" t="n">
+        <v>14288980.05949448</v>
+      </c>
+      <c r="C169" t="n">
+        <v>5951746.544758592</v>
+      </c>
+      <c r="D169" t="n">
+        <v>9375333.418723315</v>
+      </c>
+      <c r="E169" t="n">
+        <v>0</v>
+      </c>
+      <c r="F169" t="n">
+        <v>23664313.47821779</v>
+      </c>
+      <c r="G169" t="n">
+        <v>5951746.544758592</v>
+      </c>
+      <c r="H169" t="n">
+        <v>15227242.86677872</v>
+      </c>
+      <c r="I169" t="n">
+        <v>0</v>
+      </c>
+      <c r="J169" t="n">
+        <v>0</v>
+      </c>
+      <c r="K169" t="n">
+        <v>0</v>
+      </c>
+      <c r="L169" t="n">
+        <v>6074923.049917719</v>
+      </c>
+      <c r="M169" t="n">
+        <v>50918225.93967282</v>
+      </c>
+      <c r="N169" t="n">
+        <v>60756.06478760712</v>
+      </c>
+      <c r="O169" t="n">
+        <v>0</v>
+      </c>
+      <c r="P169" t="n">
+        <v>60756.06478760712</v>
+      </c>
+      <c r="Q169" t="n">
+        <v>60749.23049917654</v>
+      </c>
+      <c r="R169" t="n">
+        <v>0</v>
+      </c>
+      <c r="S169" t="n">
+        <v>0</v>
+      </c>
+      <c r="T169" t="n">
+        <v>0</v>
+      </c>
+      <c r="U169" t="n">
+        <v>6.834288431157361</v>
+      </c>
+      <c r="V169" t="n">
+        <v>8.873999834060669</v>
+      </c>
+      <c r="W169" t="n">
+        <v>50918225.93967282</v>
+      </c>
+      <c r="X169" t="n">
+        <v>50918225.93967282</v>
+      </c>
+      <c r="Y169" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z169" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA169" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB169" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC169" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD169" t="inlineStr">
+        <is>
+          <t>carbon_tax_100_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE169" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260407195125_carbon_tax_100_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="B170" t="n">
+        <v>0</v>
+      </c>
+      <c r="C170" t="n">
+        <v>0</v>
+      </c>
+      <c r="D170" t="n">
+        <v>0</v>
+      </c>
+      <c r="E170" t="n">
+        <v>0</v>
+      </c>
+      <c r="F170" t="n">
+        <v>0</v>
+      </c>
+      <c r="G170" t="n">
+        <v>0</v>
+      </c>
+      <c r="H170" t="n">
+        <v>0</v>
+      </c>
+      <c r="I170" t="n">
+        <v>0</v>
+      </c>
+      <c r="J170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K170" t="n">
+        <v>0</v>
+      </c>
+      <c r="L170" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="M170" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="N170" t="n">
+        <v>607492.3049917679</v>
+      </c>
+      <c r="O170" t="n">
+        <v>0</v>
+      </c>
+      <c r="P170" t="n">
+        <v>607492.3049917679</v>
+      </c>
+      <c r="Q170" t="n">
+        <v>607492.3049917654</v>
+      </c>
+      <c r="R170" t="n">
+        <v>0</v>
+      </c>
+      <c r="S170" t="n">
+        <v>0</v>
+      </c>
+      <c r="T170" t="n">
+        <v>0</v>
+      </c>
+      <c r="U170" t="n">
+        <v>0</v>
+      </c>
+      <c r="V170" t="n">
+        <v>26.71300005912781</v>
+      </c>
+      <c r="W170" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="X170" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="Y170" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z170" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA170" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB170" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC170" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD170" t="inlineStr">
+        <is>
+          <t>carbon_tax_100_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE170" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260407195432_carbon_tax_100_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="B171" t="n">
+        <v>0</v>
+      </c>
+      <c r="C171" t="n">
+        <v>0</v>
+      </c>
+      <c r="D171" t="n">
+        <v>0</v>
+      </c>
+      <c r="E171" t="n">
+        <v>0</v>
+      </c>
+      <c r="F171" t="n">
+        <v>0</v>
+      </c>
+      <c r="G171" t="n">
+        <v>0</v>
+      </c>
+      <c r="H171" t="n">
+        <v>0</v>
+      </c>
+      <c r="I171" t="n">
+        <v>0</v>
+      </c>
+      <c r="J171" t="n">
+        <v>0</v>
+      </c>
+      <c r="K171" t="n">
+        <v>0</v>
+      </c>
+      <c r="L171" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="M171" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="N171" t="n">
+        <v>607492.3049917679</v>
+      </c>
+      <c r="O171" t="n">
+        <v>0</v>
+      </c>
+      <c r="P171" t="n">
+        <v>607492.3049917679</v>
+      </c>
+      <c r="Q171" t="n">
+        <v>607492.3049917654</v>
+      </c>
+      <c r="R171" t="n">
+        <v>0</v>
+      </c>
+      <c r="S171" t="n">
+        <v>0</v>
+      </c>
+      <c r="T171" t="n">
+        <v>0</v>
+      </c>
+      <c r="U171" t="n">
+        <v>0</v>
+      </c>
+      <c r="V171" t="n">
+        <v>22.51099991798401</v>
+      </c>
+      <c r="W171" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="X171" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="Y171" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z171" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA171" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB171" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC171" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD171" t="inlineStr">
+        <is>
+          <t>carbon_tax_100_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE171" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260407195752_carbon_tax_100_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="B172" t="n">
+        <v>0</v>
+      </c>
+      <c r="C172" t="n">
+        <v>0</v>
+      </c>
+      <c r="D172" t="n">
+        <v>0</v>
+      </c>
+      <c r="E172" t="n">
+        <v>0</v>
+      </c>
+      <c r="F172" t="n">
+        <v>0</v>
+      </c>
+      <c r="G172" t="n">
+        <v>0</v>
+      </c>
+      <c r="H172" t="n">
+        <v>0</v>
+      </c>
+      <c r="I172" t="n">
+        <v>0</v>
+      </c>
+      <c r="J172" t="n">
+        <v>0</v>
+      </c>
+      <c r="K172" t="n">
+        <v>0</v>
+      </c>
+      <c r="L172" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="M172" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="N172" t="n">
+        <v>607492.3049917679</v>
+      </c>
+      <c r="O172" t="n">
+        <v>0</v>
+      </c>
+      <c r="P172" t="n">
+        <v>607492.3049917679</v>
+      </c>
+      <c r="Q172" t="n">
+        <v>607492.3049917654</v>
+      </c>
+      <c r="R172" t="n">
+        <v>0</v>
+      </c>
+      <c r="S172" t="n">
+        <v>0</v>
+      </c>
+      <c r="T172" t="n">
+        <v>0</v>
+      </c>
+      <c r="U172" t="n">
+        <v>0</v>
+      </c>
+      <c r="V172" t="n">
+        <v>19.82000017166138</v>
+      </c>
+      <c r="W172" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="X172" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="Y172" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z172" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA172" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB172" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC172" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD172" t="inlineStr">
+        <is>
+          <t>carbon_tax_100_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE172" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260407200121_carbon_tax_100_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="B173" t="n">
+        <v>0</v>
+      </c>
+      <c r="C173" t="n">
+        <v>0</v>
+      </c>
+      <c r="D173" t="n">
+        <v>0</v>
+      </c>
+      <c r="E173" t="n">
+        <v>0</v>
+      </c>
+      <c r="F173" t="n">
+        <v>0</v>
+      </c>
+      <c r="G173" t="n">
+        <v>0</v>
+      </c>
+      <c r="H173" t="n">
+        <v>0</v>
+      </c>
+      <c r="I173" t="n">
+        <v>0</v>
+      </c>
+      <c r="J173" t="n">
+        <v>0</v>
+      </c>
+      <c r="K173" t="n">
+        <v>0</v>
+      </c>
+      <c r="L173" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="M173" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="N173" t="n">
+        <v>607492.3049917679</v>
+      </c>
+      <c r="O173" t="n">
+        <v>0</v>
+      </c>
+      <c r="P173" t="n">
+        <v>607492.3049917679</v>
+      </c>
+      <c r="Q173" t="n">
+        <v>607492.3049917654</v>
+      </c>
+      <c r="R173" t="n">
+        <v>0</v>
+      </c>
+      <c r="S173" t="n">
+        <v>0</v>
+      </c>
+      <c r="T173" t="n">
+        <v>0</v>
+      </c>
+      <c r="U173" t="n">
+        <v>0</v>
+      </c>
+      <c r="V173" t="n">
+        <v>18.19799995422363</v>
+      </c>
+      <c r="W173" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="X173" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="Y173" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z173" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA173" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB173" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC173" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD173" t="inlineStr">
+        <is>
+          <t>carbon_tax_100_el_price_250</t>
+        </is>
+      </c>
+      <c r="AE173" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260407200429_carbon_tax_100_el_price_250</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="n">
+        <v>53955687.46463151</v>
+      </c>
+      <c r="B174" t="n">
+        <v>14288980.05949448</v>
+      </c>
+      <c r="C174" t="n">
+        <v>5951746.544758592</v>
+      </c>
+      <c r="D174" t="n">
+        <v>9375333.418723315</v>
+      </c>
+      <c r="E174" t="n">
+        <v>0</v>
+      </c>
+      <c r="F174" t="n">
+        <v>23664313.47821779</v>
+      </c>
+      <c r="G174" t="n">
+        <v>5951746.544758592</v>
+      </c>
+      <c r="H174" t="n">
+        <v>15227242.86677872</v>
+      </c>
+      <c r="I174" t="n">
+        <v>0</v>
+      </c>
+      <c r="J174" t="n">
+        <v>0</v>
+      </c>
+      <c r="K174" t="n">
+        <v>0</v>
+      </c>
+      <c r="L174" t="n">
+        <v>9112384.574876415</v>
+      </c>
+      <c r="M174" t="n">
+        <v>53955687.46463151</v>
+      </c>
+      <c r="N174" t="n">
+        <v>60756.06478760712</v>
+      </c>
+      <c r="O174" t="n">
+        <v>0</v>
+      </c>
+      <c r="P174" t="n">
+        <v>60756.06478760712</v>
+      </c>
+      <c r="Q174" t="n">
+        <v>60749.23049917654</v>
+      </c>
+      <c r="R174" t="n">
+        <v>0</v>
+      </c>
+      <c r="S174" t="n">
+        <v>0</v>
+      </c>
+      <c r="T174" t="n">
+        <v>0</v>
+      </c>
+      <c r="U174" t="n">
+        <v>6.834288431157361</v>
+      </c>
+      <c r="V174" t="n">
+        <v>16.90799999237061</v>
+      </c>
+      <c r="W174" t="n">
+        <v>53090238.47230982</v>
+      </c>
+      <c r="X174" t="n">
+        <v>53955687.46463151</v>
+      </c>
+      <c r="Y174" t="n">
+        <v>865448.9923216924</v>
+      </c>
+      <c r="Z174" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA174" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB174" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC174" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD174" t="inlineStr">
+        <is>
+          <t>carbon_tax_150_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE174" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260407200744_carbon_tax_150_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="n">
+        <v>66962942.61964789</v>
+      </c>
+      <c r="B175" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C175" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="D175" t="n">
+        <v>27323116.73979999</v>
+      </c>
+      <c r="E175" t="n">
+        <v>0</v>
+      </c>
+      <c r="F175" t="n">
+        <v>44968491.63269459</v>
+      </c>
+      <c r="G175" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="H175" t="n">
+        <v>14183168.38067319</v>
+      </c>
+      <c r="I175" t="n">
+        <v>0</v>
+      </c>
+      <c r="J175" t="n">
+        <v>0</v>
+      </c>
+      <c r="K175" t="n">
+        <v>0</v>
+      </c>
+      <c r="L175" t="n">
+        <v>1085645.259932396</v>
+      </c>
+      <c r="M175" t="n">
+        <v>66962942.61964789</v>
+      </c>
+      <c r="N175" t="n">
+        <v>7245.844635991023</v>
+      </c>
+      <c r="O175" t="n">
+        <v>0</v>
+      </c>
+      <c r="P175" t="n">
+        <v>7245.844635991023</v>
+      </c>
+      <c r="Q175" t="n">
+        <v>7237.635066215884</v>
+      </c>
+      <c r="R175" t="n">
+        <v>0</v>
+      </c>
+      <c r="S175" t="n">
+        <v>0</v>
+      </c>
+      <c r="T175" t="n">
+        <v>0</v>
+      </c>
+      <c r="U175" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V175" t="n">
+        <v>22.99300003051758</v>
+      </c>
+      <c r="W175" t="n">
+        <v>66962942.6196409</v>
+      </c>
+      <c r="X175" t="n">
+        <v>66962942.61964789</v>
+      </c>
+      <c r="Y175" t="n">
+        <v>6.988644599914551e-06</v>
+      </c>
+      <c r="Z175" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA175" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB175" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC175" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD175" t="inlineStr">
+        <is>
+          <t>carbon_tax_150_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE175" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260407201105_carbon_tax_150_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>72836330.64776947</v>
+      </c>
+      <c r="B176" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C176" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="D176" t="n">
+        <v>27323116.73979999</v>
+      </c>
+      <c r="E176" t="n">
+        <v>0</v>
+      </c>
+      <c r="F176" t="n">
+        <v>44968491.63269459</v>
+      </c>
+      <c r="G176" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="H176" t="n">
+        <v>20056556.40879477</v>
+      </c>
+      <c r="I176" t="n">
+        <v>0</v>
+      </c>
+      <c r="J176" t="n">
+        <v>0</v>
+      </c>
+      <c r="K176" t="n">
+        <v>0</v>
+      </c>
+      <c r="L176" t="n">
+        <v>1085645.259932396</v>
+      </c>
+      <c r="M176" t="n">
+        <v>72836330.64776947</v>
+      </c>
+      <c r="N176" t="n">
+        <v>7245.844635991023</v>
+      </c>
+      <c r="O176" t="n">
+        <v>0</v>
+      </c>
+      <c r="P176" t="n">
+        <v>7245.844635991023</v>
+      </c>
+      <c r="Q176" t="n">
+        <v>7237.635066215884</v>
+      </c>
+      <c r="R176" t="n">
+        <v>0</v>
+      </c>
+      <c r="S176" t="n">
+        <v>0</v>
+      </c>
+      <c r="T176" t="n">
+        <v>0</v>
+      </c>
+      <c r="U176" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V176" t="n">
+        <v>20.2590000629425</v>
+      </c>
+      <c r="W176" t="n">
+        <v>72836330.64776246</v>
+      </c>
+      <c r="X176" t="n">
+        <v>72836330.64776947</v>
+      </c>
+      <c r="Y176" t="n">
+        <v>7.003545761108398e-06</v>
+      </c>
+      <c r="Z176" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA176" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB176" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC176" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD176" t="inlineStr">
+        <is>
+          <t>carbon_tax_150_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE176" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260407201445_carbon_tax_150_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="n">
+        <v>78132220.18272139</v>
+      </c>
+      <c r="B177" t="n">
+        <v>13228586.17399643</v>
+      </c>
+      <c r="C177" t="n">
+        <v>5758365.764824538</v>
+      </c>
+      <c r="D177" t="n">
+        <v>25517441.94529562</v>
+      </c>
+      <c r="E177" t="n">
+        <v>0</v>
+      </c>
+      <c r="F177" t="n">
+        <v>38746028.11929206</v>
+      </c>
+      <c r="G177" t="n">
+        <v>5758365.764824538</v>
+      </c>
+      <c r="H177" t="n">
+        <v>11914921.09995709</v>
+      </c>
+      <c r="I177" t="n">
+        <v>0</v>
+      </c>
+      <c r="J177" t="n">
+        <v>0</v>
+      </c>
+      <c r="K177" t="n">
+        <v>0</v>
+      </c>
+      <c r="L177" t="n">
+        <v>21712905.1986477</v>
+      </c>
+      <c r="M177" t="n">
+        <v>78132220.18272139</v>
+      </c>
+      <c r="N177" t="n">
+        <v>144759.191955763</v>
+      </c>
+      <c r="O177" t="n">
+        <v>0</v>
+      </c>
+      <c r="P177" t="n">
+        <v>144759.191955763</v>
+      </c>
+      <c r="Q177" t="n">
+        <v>144752.701324317</v>
+      </c>
+      <c r="R177" t="n">
+        <v>0</v>
+      </c>
+      <c r="S177" t="n">
+        <v>0</v>
+      </c>
+      <c r="T177" t="n">
+        <v>0</v>
+      </c>
+      <c r="U177" t="n">
+        <v>6.49063144699632</v>
+      </c>
+      <c r="V177" t="n">
+        <v>17.95300006866455</v>
+      </c>
+      <c r="W177" t="n">
+        <v>78132220.18271443</v>
+      </c>
+      <c r="X177" t="n">
+        <v>78132220.18272139</v>
+      </c>
+      <c r="Y177" t="n">
+        <v>6.958842277526855e-06</v>
+      </c>
+      <c r="Z177" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA177" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB177" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC177" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD177" t="inlineStr">
+        <is>
+          <t>carbon_tax_150_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE177" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260407201727_carbon_tax_150_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>80501852.37660313</v>
+      </c>
+      <c r="B178" t="n">
+        <v>13228586.17399643</v>
+      </c>
+      <c r="C178" t="n">
+        <v>5758365.764824538</v>
+      </c>
+      <c r="D178" t="n">
+        <v>25517441.94529562</v>
+      </c>
+      <c r="E178" t="n">
+        <v>0</v>
+      </c>
+      <c r="F178" t="n">
+        <v>38746028.11929206</v>
+      </c>
+      <c r="G178" t="n">
+        <v>5758365.764824538</v>
+      </c>
+      <c r="H178" t="n">
+        <v>14284553.29383882</v>
+      </c>
+      <c r="I178" t="n">
+        <v>0</v>
+      </c>
+      <c r="J178" t="n">
+        <v>0</v>
+      </c>
+      <c r="K178" t="n">
+        <v>0</v>
+      </c>
+      <c r="L178" t="n">
+        <v>21712905.1986477</v>
+      </c>
+      <c r="M178" t="n">
+        <v>80501852.37660313</v>
+      </c>
+      <c r="N178" t="n">
+        <v>144759.191955763</v>
+      </c>
+      <c r="O178" t="n">
+        <v>0</v>
+      </c>
+      <c r="P178" t="n">
+        <v>144759.191955763</v>
+      </c>
+      <c r="Q178" t="n">
+        <v>144752.701324317</v>
+      </c>
+      <c r="R178" t="n">
+        <v>0</v>
+      </c>
+      <c r="S178" t="n">
+        <v>0</v>
+      </c>
+      <c r="T178" t="n">
+        <v>0</v>
+      </c>
+      <c r="U178" t="n">
+        <v>6.49063144699632</v>
+      </c>
+      <c r="V178" t="n">
+        <v>17.3490002155304</v>
+      </c>
+      <c r="W178" t="n">
+        <v>80501852.37659612</v>
+      </c>
+      <c r="X178" t="n">
+        <v>80501852.37660313</v>
+      </c>
+      <c r="Y178" t="n">
+        <v>7.003545761108398e-06</v>
+      </c>
+      <c r="Z178" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA178" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB178" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC178" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD178" t="inlineStr">
+        <is>
+          <t>carbon_tax_150_el_price_250</t>
+        </is>
+      </c>
+      <c r="AE178" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260407202116_carbon_tax_150_el_price_250</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="n">
+        <v>56993148.98959054</v>
+      </c>
+      <c r="B179" t="n">
+        <v>14288980.05949448</v>
+      </c>
+      <c r="C179" t="n">
+        <v>5951746.544758592</v>
+      </c>
+      <c r="D179" t="n">
+        <v>9375333.418723315</v>
+      </c>
+      <c r="E179" t="n">
+        <v>0</v>
+      </c>
+      <c r="F179" t="n">
+        <v>23664313.47821779</v>
+      </c>
+      <c r="G179" t="n">
+        <v>5951746.544758592</v>
+      </c>
+      <c r="H179" t="n">
+        <v>15227242.86677872</v>
+      </c>
+      <c r="I179" t="n">
+        <v>0</v>
+      </c>
+      <c r="J179" t="n">
+        <v>0</v>
+      </c>
+      <c r="K179" t="n">
+        <v>0</v>
+      </c>
+      <c r="L179" t="n">
+        <v>12149846.09983544</v>
+      </c>
+      <c r="M179" t="n">
+        <v>56993148.98959054</v>
+      </c>
+      <c r="N179" t="n">
+        <v>60756.06478760712</v>
+      </c>
+      <c r="O179" t="n">
+        <v>0</v>
+      </c>
+      <c r="P179" t="n">
+        <v>60756.06478760712</v>
+      </c>
+      <c r="Q179" t="n">
+        <v>60749.23049917654</v>
+      </c>
+      <c r="R179" t="n">
+        <v>0</v>
+      </c>
+      <c r="S179" t="n">
+        <v>0</v>
+      </c>
+      <c r="T179" t="n">
+        <v>0</v>
+      </c>
+      <c r="U179" t="n">
+        <v>6.834288431157361</v>
+      </c>
+      <c r="V179" t="n">
+        <v>17.73799991607666</v>
+      </c>
+      <c r="W179" t="n">
+        <v>56993148.98959054</v>
+      </c>
+      <c r="X179" t="n">
+        <v>56993148.98959054</v>
+      </c>
+      <c r="Y179" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z179" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA179" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB179" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC179" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD179" t="inlineStr">
+        <is>
+          <t>carbon_tax_200_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE179" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260407202356_carbon_tax_200_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="n">
+        <v>67324824.3729587</v>
+      </c>
+      <c r="B180" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C180" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="D180" t="n">
+        <v>27323116.73979999</v>
+      </c>
+      <c r="E180" t="n">
+        <v>0</v>
+      </c>
+      <c r="F180" t="n">
+        <v>44968491.63269459</v>
+      </c>
+      <c r="G180" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="H180" t="n">
+        <v>14183168.38067319</v>
+      </c>
+      <c r="I180" t="n">
+        <v>0</v>
+      </c>
+      <c r="J180" t="n">
+        <v>0</v>
+      </c>
+      <c r="K180" t="n">
+        <v>0</v>
+      </c>
+      <c r="L180" t="n">
+        <v>1447527.013243217</v>
+      </c>
+      <c r="M180" t="n">
+        <v>67324824.3729587</v>
+      </c>
+      <c r="N180" t="n">
+        <v>7245.844635991128</v>
+      </c>
+      <c r="O180" t="n">
+        <v>0</v>
+      </c>
+      <c r="P180" t="n">
+        <v>7245.844635991128</v>
+      </c>
+      <c r="Q180" t="n">
+        <v>7237.635066215956</v>
+      </c>
+      <c r="R180" t="n">
+        <v>0</v>
+      </c>
+      <c r="S180" t="n">
+        <v>0</v>
+      </c>
+      <c r="T180" t="n">
+        <v>0</v>
+      </c>
+      <c r="U180" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V180" t="n">
+        <v>21.35000014305115</v>
+      </c>
+      <c r="W180" t="n">
+        <v>67324824.3729587</v>
+      </c>
+      <c r="X180" t="n">
+        <v>67324824.3729587</v>
+      </c>
+      <c r="Y180" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z180" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA180" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB180" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC180" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD180" t="inlineStr">
+        <is>
+          <t>carbon_tax_200_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE180" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260407202800_carbon_tax_200_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="n">
+        <v>73198212.40108028</v>
+      </c>
+      <c r="B181" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C181" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="D181" t="n">
+        <v>27323116.73979999</v>
+      </c>
+      <c r="E181" t="n">
+        <v>0</v>
+      </c>
+      <c r="F181" t="n">
+        <v>44968491.63269459</v>
+      </c>
+      <c r="G181" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="H181" t="n">
+        <v>20056556.40879477</v>
+      </c>
+      <c r="I181" t="n">
+        <v>0</v>
+      </c>
+      <c r="J181" t="n">
+        <v>0</v>
+      </c>
+      <c r="K181" t="n">
+        <v>0</v>
+      </c>
+      <c r="L181" t="n">
+        <v>1447527.013243219</v>
+      </c>
+      <c r="M181" t="n">
+        <v>73198212.40108028</v>
+      </c>
+      <c r="N181" t="n">
+        <v>7245.844635991135</v>
+      </c>
+      <c r="O181" t="n">
+        <v>0</v>
+      </c>
+      <c r="P181" t="n">
+        <v>7245.844635991135</v>
+      </c>
+      <c r="Q181" t="n">
+        <v>7237.63506621596</v>
+      </c>
+      <c r="R181" t="n">
+        <v>0</v>
+      </c>
+      <c r="S181" t="n">
+        <v>0</v>
+      </c>
+      <c r="T181" t="n">
+        <v>0</v>
+      </c>
+      <c r="U181" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V181" t="n">
+        <v>18.52800011634827</v>
+      </c>
+      <c r="W181" t="n">
+        <v>73198212.40108028</v>
+      </c>
+      <c r="X181" t="n">
+        <v>73198212.40108028</v>
+      </c>
+      <c r="Y181" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z181" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA181" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB181" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC181" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD181" t="inlineStr">
+        <is>
+          <t>carbon_tax_200_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE181" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260407203046_carbon_tax_200_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>79071600.42920169</v>
+      </c>
+      <c r="B182" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C182" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="D182" t="n">
+        <v>27323116.73979999</v>
+      </c>
+      <c r="E182" t="n">
+        <v>0</v>
+      </c>
+      <c r="F182" t="n">
+        <v>44968491.63269459</v>
+      </c>
+      <c r="G182" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="H182" t="n">
+        <v>25929944.43691619</v>
+      </c>
+      <c r="I182" t="n">
+        <v>0</v>
+      </c>
+      <c r="J182" t="n">
+        <v>0</v>
+      </c>
+      <c r="K182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L182" t="n">
+        <v>1447527.013243193</v>
+      </c>
+      <c r="M182" t="n">
+        <v>79071600.42920169</v>
+      </c>
+      <c r="N182" t="n">
+        <v>7245.844635991023</v>
+      </c>
+      <c r="O182" t="n">
+        <v>0</v>
+      </c>
+      <c r="P182" t="n">
+        <v>7245.844635991023</v>
+      </c>
+      <c r="Q182" t="n">
+        <v>7237.635066215884</v>
+      </c>
+      <c r="R182" t="n">
+        <v>0</v>
+      </c>
+      <c r="S182" t="n">
+        <v>0</v>
+      </c>
+      <c r="T182" t="n">
+        <v>0</v>
+      </c>
+      <c r="U182" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V182" t="n">
+        <v>19.75300002098083</v>
+      </c>
+      <c r="W182" t="n">
+        <v>79071600.42920169</v>
+      </c>
+      <c r="X182" t="n">
+        <v>79071600.42920169</v>
+      </c>
+      <c r="Y182" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z182" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA182" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB182" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC182" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD182" t="inlineStr">
+        <is>
+          <t>carbon_tax_200_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE182" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260407203507_carbon_tax_200_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>84944988.45732322</v>
+      </c>
+      <c r="B183" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C183" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="D183" t="n">
+        <v>27323116.73979999</v>
+      </c>
+      <c r="E183" t="n">
+        <v>0</v>
+      </c>
+      <c r="F183" t="n">
+        <v>44968491.63269459</v>
+      </c>
+      <c r="G183" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="H183" t="n">
+        <v>31803332.46503772</v>
+      </c>
+      <c r="I183" t="n">
+        <v>0</v>
+      </c>
+      <c r="J183" t="n">
+        <v>0</v>
+      </c>
+      <c r="K183" t="n">
+        <v>0</v>
+      </c>
+      <c r="L183" t="n">
+        <v>1447527.013243193</v>
+      </c>
+      <c r="M183" t="n">
+        <v>84944988.45732322</v>
+      </c>
+      <c r="N183" t="n">
+        <v>7245.844635991023</v>
+      </c>
+      <c r="O183" t="n">
+        <v>0</v>
+      </c>
+      <c r="P183" t="n">
+        <v>7245.844635991023</v>
+      </c>
+      <c r="Q183" t="n">
+        <v>7237.635066215884</v>
+      </c>
+      <c r="R183" t="n">
+        <v>0</v>
+      </c>
+      <c r="S183" t="n">
+        <v>0</v>
+      </c>
+      <c r="T183" t="n">
+        <v>0</v>
+      </c>
+      <c r="U183" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V183" t="n">
+        <v>19.14999985694885</v>
+      </c>
+      <c r="W183" t="n">
+        <v>84944988.45732322</v>
+      </c>
+      <c r="X183" t="n">
+        <v>84944988.45732322</v>
+      </c>
+      <c r="Y183" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z183" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA183" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB183" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC183" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD183" t="inlineStr">
+        <is>
+          <t>carbon_tax_200_el_price_250</t>
+        </is>
+      </c>
+      <c r="AE183" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260407203750_carbon_tax_200_el_price_250</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="n">
+        <v>60030610.51454906</v>
+      </c>
+      <c r="B184" t="n">
+        <v>14288980.05949448</v>
+      </c>
+      <c r="C184" t="n">
+        <v>5951746.544758592</v>
+      </c>
+      <c r="D184" t="n">
+        <v>9375333.418723315</v>
+      </c>
+      <c r="E184" t="n">
+        <v>0</v>
+      </c>
+      <c r="F184" t="n">
+        <v>23664313.47821779</v>
+      </c>
+      <c r="G184" t="n">
+        <v>5951746.544758592</v>
+      </c>
+      <c r="H184" t="n">
+        <v>15227242.86677872</v>
+      </c>
+      <c r="I184" t="n">
+        <v>0</v>
+      </c>
+      <c r="J184" t="n">
+        <v>0</v>
+      </c>
+      <c r="K184" t="n">
+        <v>0</v>
+      </c>
+      <c r="L184" t="n">
+        <v>15187307.62479397</v>
+      </c>
+      <c r="M184" t="n">
+        <v>60030610.51454906</v>
+      </c>
+      <c r="N184" t="n">
+        <v>60756.06478760712</v>
+      </c>
+      <c r="O184" t="n">
+        <v>0</v>
+      </c>
+      <c r="P184" t="n">
+        <v>60756.06478760712</v>
+      </c>
+      <c r="Q184" t="n">
+        <v>60749.23049917654</v>
+      </c>
+      <c r="R184" t="n">
+        <v>0</v>
+      </c>
+      <c r="S184" t="n">
+        <v>0</v>
+      </c>
+      <c r="T184" t="n">
+        <v>0</v>
+      </c>
+      <c r="U184" t="n">
+        <v>6.834288431157361</v>
+      </c>
+      <c r="V184" t="n">
+        <v>17.87800002098083</v>
+      </c>
+      <c r="W184" t="n">
+        <v>60030610.51454906</v>
+      </c>
+      <c r="X184" t="n">
+        <v>60030610.51454906</v>
+      </c>
+      <c r="Y184" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z184" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA184" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB184" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC184" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD184" t="inlineStr">
+        <is>
+          <t>carbon_tax_250_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE184" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260407204035_carbon_tax_250_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>67686706.1262694</v>
+      </c>
+      <c r="B185" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C185" t="n">
+        <v>6725637.346347711</v>
+      </c>
+      <c r="D185" t="n">
+        <v>27323116.73979999</v>
+      </c>
+      <c r="E185" t="n">
+        <v>0</v>
+      </c>
+      <c r="F185" t="n">
+        <v>44968491.63269459</v>
+      </c>
+      <c r="G185" t="n">
+        <v>6725637.346347711</v>
+      </c>
+      <c r="H185" t="n">
+        <v>14183168.38067319</v>
+      </c>
+      <c r="I185" t="n">
+        <v>0</v>
+      </c>
+      <c r="J185" t="n">
+        <v>0</v>
+      </c>
+      <c r="K185" t="n">
+        <v>0</v>
+      </c>
+      <c r="L185" t="n">
+        <v>1809408.766553909</v>
+      </c>
+      <c r="M185" t="n">
+        <v>67686706.1262694</v>
+      </c>
+      <c r="N185" t="n">
+        <v>7245.844635990867</v>
+      </c>
+      <c r="O185" t="n">
+        <v>0</v>
+      </c>
+      <c r="P185" t="n">
+        <v>7245.844635990867</v>
+      </c>
+      <c r="Q185" t="n">
+        <v>7237.63506621584</v>
+      </c>
+      <c r="R185" t="n">
+        <v>0</v>
+      </c>
+      <c r="S185" t="n">
+        <v>0</v>
+      </c>
+      <c r="T185" t="n">
+        <v>0</v>
+      </c>
+      <c r="U185" t="n">
+        <v>8.209569775222588</v>
+      </c>
+      <c r="V185" t="n">
+        <v>23.11500000953674</v>
+      </c>
+      <c r="W185" t="n">
+        <v>67686706.1262694</v>
+      </c>
+      <c r="X185" t="n">
+        <v>67686706.1262694</v>
+      </c>
+      <c r="Y185" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z185" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA185" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB185" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC185" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD185" t="inlineStr">
+        <is>
+          <t>carbon_tax_250_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE185" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260407204517_carbon_tax_250_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>73560094.15439105</v>
+      </c>
+      <c r="B186" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C186" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="D186" t="n">
+        <v>27323116.73979999</v>
+      </c>
+      <c r="E186" t="n">
+        <v>0</v>
+      </c>
+      <c r="F186" t="n">
+        <v>44968491.63269459</v>
+      </c>
+      <c r="G186" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="H186" t="n">
+        <v>20056556.40879477</v>
+      </c>
+      <c r="I186" t="n">
+        <v>0</v>
+      </c>
+      <c r="J186" t="n">
+        <v>0</v>
+      </c>
+      <c r="K186" t="n">
+        <v>0</v>
+      </c>
+      <c r="L186" t="n">
+        <v>1809408.766553984</v>
+      </c>
+      <c r="M186" t="n">
+        <v>73560094.15439105</v>
+      </c>
+      <c r="N186" t="n">
+        <v>7245.844635991149</v>
+      </c>
+      <c r="O186" t="n">
+        <v>0</v>
+      </c>
+      <c r="P186" t="n">
+        <v>7245.844635991149</v>
+      </c>
+      <c r="Q186" t="n">
+        <v>7237.635066215972</v>
+      </c>
+      <c r="R186" t="n">
+        <v>0</v>
+      </c>
+      <c r="S186" t="n">
+        <v>0</v>
+      </c>
+      <c r="T186" t="n">
+        <v>0</v>
+      </c>
+      <c r="U186" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V186" t="n">
+        <v>20.09999990463257</v>
+      </c>
+      <c r="W186" t="n">
+        <v>73560094.15439105</v>
+      </c>
+      <c r="X186" t="n">
+        <v>73560094.15439105</v>
+      </c>
+      <c r="Y186" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z186" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA186" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB186" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC186" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD186" t="inlineStr">
+        <is>
+          <t>carbon_tax_250_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE186" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260407204805_carbon_tax_250_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>79433482.18251243</v>
+      </c>
+      <c r="B187" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C187" t="n">
+        <v>6725637.34634771</v>
+      </c>
+      <c r="D187" t="n">
+        <v>27323116.73979999</v>
+      </c>
+      <c r="E187" t="n">
+        <v>0</v>
+      </c>
+      <c r="F187" t="n">
+        <v>44968491.63269459</v>
+      </c>
+      <c r="G187" t="n">
+        <v>6725637.34634771</v>
+      </c>
+      <c r="H187" t="n">
+        <v>25929944.4369162</v>
+      </c>
+      <c r="I187" t="n">
+        <v>0</v>
+      </c>
+      <c r="J187" t="n">
+        <v>0</v>
+      </c>
+      <c r="K187" t="n">
+        <v>0</v>
+      </c>
+      <c r="L187" t="n">
+        <v>1809408.766553939</v>
+      </c>
+      <c r="M187" t="n">
+        <v>79433482.18251243</v>
+      </c>
+      <c r="N187" t="n">
+        <v>7245.844635991052</v>
+      </c>
+      <c r="O187" t="n">
+        <v>0</v>
+      </c>
+      <c r="P187" t="n">
+        <v>7245.844635991052</v>
+      </c>
+      <c r="Q187" t="n">
+        <v>7237.63506621566</v>
+      </c>
+      <c r="R187" t="n">
+        <v>0</v>
+      </c>
+      <c r="S187" t="n">
+        <v>0</v>
+      </c>
+      <c r="T187" t="n">
+        <v>0</v>
+      </c>
+      <c r="U187" t="n">
+        <v>8.209569775222587</v>
+      </c>
+      <c r="V187" t="n">
+        <v>19.68499994277954</v>
+      </c>
+      <c r="W187" t="n">
+        <v>79433482.18251243</v>
+      </c>
+      <c r="X187" t="n">
+        <v>79433482.18251243</v>
+      </c>
+      <c r="Y187" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z187" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA187" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB187" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC187" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD187" t="inlineStr">
+        <is>
+          <t>carbon_tax_250_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE187" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260407205050_carbon_tax_250_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>85306870.21063398</v>
+      </c>
+      <c r="B188" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C188" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="D188" t="n">
+        <v>27323116.73979999</v>
+      </c>
+      <c r="E188" t="n">
+        <v>0</v>
+      </c>
+      <c r="F188" t="n">
+        <v>44968491.63269459</v>
+      </c>
+      <c r="G188" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="H188" t="n">
+        <v>31803332.46503772</v>
+      </c>
+      <c r="I188" t="n">
+        <v>0</v>
+      </c>
+      <c r="J188" t="n">
+        <v>0</v>
+      </c>
+      <c r="K188" t="n">
+        <v>0</v>
+      </c>
+      <c r="L188" t="n">
+        <v>1809408.766553953</v>
+      </c>
+      <c r="M188" t="n">
+        <v>85306870.21063398</v>
+      </c>
+      <c r="N188" t="n">
+        <v>7245.844635991023</v>
+      </c>
+      <c r="O188" t="n">
+        <v>0</v>
+      </c>
+      <c r="P188" t="n">
+        <v>7245.844635991023</v>
+      </c>
+      <c r="Q188" t="n">
+        <v>7237.635066215884</v>
+      </c>
+      <c r="R188" t="n">
+        <v>0</v>
+      </c>
+      <c r="S188" t="n">
+        <v>0</v>
+      </c>
+      <c r="T188" t="n">
+        <v>0</v>
+      </c>
+      <c r="U188" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V188" t="n">
+        <v>24.50999999046326</v>
+      </c>
+      <c r="W188" t="n">
+        <v>85306870.21063398</v>
+      </c>
+      <c r="X188" t="n">
+        <v>85306870.21063398</v>
+      </c>
+      <c r="Y188" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z188" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA188" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB188" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC188" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD188" t="inlineStr">
+        <is>
+          <t>carbon_tax_250_el_price_250</t>
+        </is>
+      </c>
+      <c r="AE188" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260407205333_carbon_tax_250_el_price_250</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>62175199.85145879</v>
+      </c>
+      <c r="B189" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C189" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="D189" t="n">
+        <v>27323116.73979999</v>
+      </c>
+      <c r="E189" t="n">
+        <v>0</v>
+      </c>
+      <c r="F189" t="n">
+        <v>44968491.63269459</v>
+      </c>
+      <c r="G189" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="H189" t="n">
+        <v>8309780.352551687</v>
+      </c>
+      <c r="I189" t="n">
+        <v>0</v>
+      </c>
+      <c r="J189" t="n">
+        <v>0</v>
+      </c>
+      <c r="K189" t="n">
+        <v>0</v>
+      </c>
+      <c r="L189" t="n">
+        <v>2171290.519864813</v>
+      </c>
+      <c r="M189" t="n">
+        <v>62175199.85145879</v>
+      </c>
+      <c r="N189" t="n">
+        <v>7245.844635991104</v>
+      </c>
+      <c r="O189" t="n">
+        <v>0</v>
+      </c>
+      <c r="P189" t="n">
+        <v>7245.844635991104</v>
+      </c>
+      <c r="Q189" t="n">
+        <v>7237.635066215933</v>
+      </c>
+      <c r="R189" t="n">
+        <v>0</v>
+      </c>
+      <c r="S189" t="n">
+        <v>0</v>
+      </c>
+      <c r="T189" t="n">
+        <v>0</v>
+      </c>
+      <c r="U189" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V189" t="n">
+        <v>17.35899996757507</v>
+      </c>
+      <c r="W189" t="n">
+        <v>62175199.85144535</v>
+      </c>
+      <c r="X189" t="n">
+        <v>62175199.85145879</v>
+      </c>
+      <c r="Y189" t="n">
+        <v>1.344084739685059e-05</v>
+      </c>
+      <c r="Z189" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA189" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB189" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC189" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD189" t="inlineStr">
+        <is>
+          <t>carbon_tax_300_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE189" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260407205853_carbon_tax_300_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="n">
+        <v>68048587.8795803</v>
+      </c>
+      <c r="B190" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C190" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="D190" t="n">
+        <v>27323116.73979999</v>
+      </c>
+      <c r="E190" t="n">
+        <v>0</v>
+      </c>
+      <c r="F190" t="n">
+        <v>44968491.63269459</v>
+      </c>
+      <c r="G190" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="H190" t="n">
+        <v>14183168.38067319</v>
+      </c>
+      <c r="I190" t="n">
+        <v>0</v>
+      </c>
+      <c r="J190" t="n">
+        <v>0</v>
+      </c>
+      <c r="K190" t="n">
+        <v>0</v>
+      </c>
+      <c r="L190" t="n">
+        <v>2171290.519864813</v>
+      </c>
+      <c r="M190" t="n">
+        <v>68048587.8795803</v>
+      </c>
+      <c r="N190" t="n">
+        <v>7245.844635991101</v>
+      </c>
+      <c r="O190" t="n">
+        <v>0</v>
+      </c>
+      <c r="P190" t="n">
+        <v>7245.844635991101</v>
+      </c>
+      <c r="Q190" t="n">
+        <v>7237.635066215942</v>
+      </c>
+      <c r="R190" t="n">
+        <v>0</v>
+      </c>
+      <c r="S190" t="n">
+        <v>0</v>
+      </c>
+      <c r="T190" t="n">
+        <v>0</v>
+      </c>
+      <c r="U190" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V190" t="n">
+        <v>23.73300004005432</v>
+      </c>
+      <c r="W190" t="n">
+        <v>68048587.87956655</v>
+      </c>
+      <c r="X190" t="n">
+        <v>68048587.8795803</v>
+      </c>
+      <c r="Y190" t="n">
+        <v>1.375377178192139e-05</v>
+      </c>
+      <c r="Z190" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA190" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB190" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC190" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD190" t="inlineStr">
+        <is>
+          <t>carbon_tax_300_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE190" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260407210136_carbon_tax_300_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="n">
+        <v>73921975.90770189</v>
+      </c>
+      <c r="B191" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C191" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="D191" t="n">
+        <v>27323116.73979999</v>
+      </c>
+      <c r="E191" t="n">
+        <v>0</v>
+      </c>
+      <c r="F191" t="n">
+        <v>44968491.63269459</v>
+      </c>
+      <c r="G191" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="H191" t="n">
+        <v>20056556.40879477</v>
+      </c>
+      <c r="I191" t="n">
+        <v>0</v>
+      </c>
+      <c r="J191" t="n">
+        <v>0</v>
+      </c>
+      <c r="K191" t="n">
+        <v>0</v>
+      </c>
+      <c r="L191" t="n">
+        <v>2171290.519864826</v>
+      </c>
+      <c r="M191" t="n">
+        <v>73921975.90770189</v>
+      </c>
+      <c r="N191" t="n">
+        <v>7245.844635991143</v>
+      </c>
+      <c r="O191" t="n">
+        <v>0</v>
+      </c>
+      <c r="P191" t="n">
+        <v>7245.844635991143</v>
+      </c>
+      <c r="Q191" t="n">
+        <v>7237.635066215969</v>
+      </c>
+      <c r="R191" t="n">
+        <v>0</v>
+      </c>
+      <c r="S191" t="n">
+        <v>0</v>
+      </c>
+      <c r="T191" t="n">
+        <v>0</v>
+      </c>
+      <c r="U191" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V191" t="n">
+        <v>21.00399994850159</v>
+      </c>
+      <c r="W191" t="n">
+        <v>73921975.90768784</v>
+      </c>
+      <c r="X191" t="n">
+        <v>73921975.90770189</v>
+      </c>
+      <c r="Y191" t="n">
+        <v>1.405179500579834e-05</v>
+      </c>
+      <c r="Z191" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA191" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB191" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC191" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD191" t="inlineStr">
+        <is>
+          <t>carbon_tax_300_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE191" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260407210423_carbon_tax_300_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="n">
+        <v>79795363.93582323</v>
+      </c>
+      <c r="B192" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C192" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="D192" t="n">
+        <v>27323116.73979999</v>
+      </c>
+      <c r="E192" t="n">
+        <v>0</v>
+      </c>
+      <c r="F192" t="n">
+        <v>44968491.63269459</v>
+      </c>
+      <c r="G192" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="H192" t="n">
+        <v>25929944.4369162</v>
+      </c>
+      <c r="I192" t="n">
+        <v>0</v>
+      </c>
+      <c r="J192" t="n">
+        <v>0</v>
+      </c>
+      <c r="K192" t="n">
+        <v>0</v>
+      </c>
+      <c r="L192" t="n">
+        <v>2171290.519864739</v>
+      </c>
+      <c r="M192" t="n">
+        <v>79795363.93582323</v>
+      </c>
+      <c r="N192" t="n">
+        <v>7245.844635991064</v>
+      </c>
+      <c r="O192" t="n">
+        <v>0</v>
+      </c>
+      <c r="P192" t="n">
+        <v>7245.844635991064</v>
+      </c>
+      <c r="Q192" t="n">
+        <v>7237.63506621573</v>
+      </c>
+      <c r="R192" t="n">
+        <v>0</v>
+      </c>
+      <c r="S192" t="n">
+        <v>0</v>
+      </c>
+      <c r="T192" t="n">
+        <v>0</v>
+      </c>
+      <c r="U192" t="n">
+        <v>8.209569775222587</v>
+      </c>
+      <c r="V192" t="n">
+        <v>21.39599990844727</v>
+      </c>
+      <c r="W192" t="n">
+        <v>79795363.93580902</v>
+      </c>
+      <c r="X192" t="n">
+        <v>79795363.93582323</v>
+      </c>
+      <c r="Y192" t="n">
+        <v>1.421570777893066e-05</v>
+      </c>
+      <c r="Z192" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA192" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB192" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC192" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD192" t="inlineStr">
+        <is>
+          <t>carbon_tax_300_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE192" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260407210709_carbon_tax_300_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="n">
+        <v>85668751.96394473</v>
+      </c>
+      <c r="B193" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C193" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="D193" t="n">
+        <v>27323116.73979999</v>
+      </c>
+      <c r="E193" t="n">
+        <v>0</v>
+      </c>
+      <c r="F193" t="n">
+        <v>44968491.63269459</v>
+      </c>
+      <c r="G193" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="H193" t="n">
+        <v>31803332.46503773</v>
+      </c>
+      <c r="I193" t="n">
+        <v>0</v>
+      </c>
+      <c r="J193" t="n">
+        <v>0</v>
+      </c>
+      <c r="K193" t="n">
+        <v>0</v>
+      </c>
+      <c r="L193" t="n">
+        <v>2171290.519864705</v>
+      </c>
+      <c r="M193" t="n">
+        <v>85668751.96394473</v>
+      </c>
+      <c r="N193" t="n">
+        <v>7245.844635991036</v>
+      </c>
+      <c r="O193" t="n">
+        <v>0</v>
+      </c>
+      <c r="P193" t="n">
+        <v>7245.844635991036</v>
+      </c>
+      <c r="Q193" t="n">
+        <v>7237.635066215663</v>
+      </c>
+      <c r="R193" t="n">
+        <v>0</v>
+      </c>
+      <c r="S193" t="n">
+        <v>0</v>
+      </c>
+      <c r="T193" t="n">
+        <v>0</v>
+      </c>
+      <c r="U193" t="n">
+        <v>8.209569775222587</v>
+      </c>
+      <c r="V193" t="n">
+        <v>21.24700021743774</v>
+      </c>
+      <c r="W193" t="n">
+        <v>85668751.96393028</v>
+      </c>
+      <c r="X193" t="n">
+        <v>85668751.96394473</v>
+      </c>
+      <c r="Y193" t="n">
+        <v>1.445412635803223e-05</v>
+      </c>
+      <c r="Z193" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA193" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB193" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC193" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD193" t="inlineStr">
+        <is>
+          <t>carbon_tax_300_el_price_250</t>
+        </is>
+      </c>
+      <c r="AE193" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260407211301_carbon_tax_300_el_price_250</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
results with updated opex var mea and oxy
</commit_message>
<xml_diff>
--- a/dataCaseStudy_Cement/raw_results/tech_selection/Summary.xlsx
+++ b/dataCaseStudy_Cement/raw_results/tech_selection/Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE229"/>
+  <dimension ref="A1:AE254"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24066,6 +24066,2581 @@
       <c r="AE229" t="inlineStr">
         <is>
           <t>dataCaseStudy_Cement\raw_results\tech_selection\20260420103601_carbon_tax_300_el_price_250</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="n">
+        <v>54078237.83032095</v>
+      </c>
+      <c r="B230" t="n">
+        <v>15828554.68961274</v>
+      </c>
+      <c r="C230" t="n">
+        <v>5951746.544758592</v>
+      </c>
+      <c r="D230" t="n">
+        <v>9950906.361202955</v>
+      </c>
+      <c r="E230" t="n">
+        <v>0</v>
+      </c>
+      <c r="F230" t="n">
+        <v>25779461.05081569</v>
+      </c>
+      <c r="G230" t="n">
+        <v>5951746.544758592</v>
+      </c>
+      <c r="H230" t="n">
+        <v>16272107.18482895</v>
+      </c>
+      <c r="I230" t="n">
+        <v>0</v>
+      </c>
+      <c r="J230" t="n">
+        <v>0</v>
+      </c>
+      <c r="K230" t="n">
+        <v>0</v>
+      </c>
+      <c r="L230" t="n">
+        <v>6074923.049917719</v>
+      </c>
+      <c r="M230" t="n">
+        <v>54078237.83032095</v>
+      </c>
+      <c r="N230" t="n">
+        <v>60756.06478760712</v>
+      </c>
+      <c r="O230" t="n">
+        <v>0</v>
+      </c>
+      <c r="P230" t="n">
+        <v>60756.06478760712</v>
+      </c>
+      <c r="Q230" t="n">
+        <v>60749.23049917654</v>
+      </c>
+      <c r="R230" t="n">
+        <v>0</v>
+      </c>
+      <c r="S230" t="n">
+        <v>0</v>
+      </c>
+      <c r="T230" t="n">
+        <v>0</v>
+      </c>
+      <c r="U230" t="n">
+        <v>6.834288431157361</v>
+      </c>
+      <c r="V230" t="n">
+        <v>14.63800001144409</v>
+      </c>
+      <c r="W230" t="n">
+        <v>53077940.87673726</v>
+      </c>
+      <c r="X230" t="n">
+        <v>54078237.83032095</v>
+      </c>
+      <c r="Y230" t="n">
+        <v>1000296.953583695</v>
+      </c>
+      <c r="Z230" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA230" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB230" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC230" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD230" t="inlineStr">
+        <is>
+          <t>carbon_tax_100_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE230" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260424174840_carbon_tax_100_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="B231" t="n">
+        <v>0</v>
+      </c>
+      <c r="C231" t="n">
+        <v>0</v>
+      </c>
+      <c r="D231" t="n">
+        <v>0</v>
+      </c>
+      <c r="E231" t="n">
+        <v>0</v>
+      </c>
+      <c r="F231" t="n">
+        <v>0</v>
+      </c>
+      <c r="G231" t="n">
+        <v>0</v>
+      </c>
+      <c r="H231" t="n">
+        <v>0</v>
+      </c>
+      <c r="I231" t="n">
+        <v>0</v>
+      </c>
+      <c r="J231" t="n">
+        <v>0</v>
+      </c>
+      <c r="K231" t="n">
+        <v>0</v>
+      </c>
+      <c r="L231" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="M231" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="N231" t="n">
+        <v>607492.3049917679</v>
+      </c>
+      <c r="O231" t="n">
+        <v>0</v>
+      </c>
+      <c r="P231" t="n">
+        <v>607492.3049917679</v>
+      </c>
+      <c r="Q231" t="n">
+        <v>607492.3049917654</v>
+      </c>
+      <c r="R231" t="n">
+        <v>0</v>
+      </c>
+      <c r="S231" t="n">
+        <v>0</v>
+      </c>
+      <c r="T231" t="n">
+        <v>0</v>
+      </c>
+      <c r="U231" t="n">
+        <v>0</v>
+      </c>
+      <c r="V231" t="n">
+        <v>30.37100005149841</v>
+      </c>
+      <c r="W231" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="X231" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="Y231" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z231" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA231" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB231" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC231" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD231" t="inlineStr">
+        <is>
+          <t>carbon_tax_100_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE231" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260424175211_carbon_tax_100_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="B232" t="n">
+        <v>0</v>
+      </c>
+      <c r="C232" t="n">
+        <v>0</v>
+      </c>
+      <c r="D232" t="n">
+        <v>0</v>
+      </c>
+      <c r="E232" t="n">
+        <v>0</v>
+      </c>
+      <c r="F232" t="n">
+        <v>0</v>
+      </c>
+      <c r="G232" t="n">
+        <v>0</v>
+      </c>
+      <c r="H232" t="n">
+        <v>0</v>
+      </c>
+      <c r="I232" t="n">
+        <v>0</v>
+      </c>
+      <c r="J232" t="n">
+        <v>0</v>
+      </c>
+      <c r="K232" t="n">
+        <v>0</v>
+      </c>
+      <c r="L232" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="M232" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="N232" t="n">
+        <v>607492.3049917679</v>
+      </c>
+      <c r="O232" t="n">
+        <v>0</v>
+      </c>
+      <c r="P232" t="n">
+        <v>607492.3049917679</v>
+      </c>
+      <c r="Q232" t="n">
+        <v>607492.3049917654</v>
+      </c>
+      <c r="R232" t="n">
+        <v>0</v>
+      </c>
+      <c r="S232" t="n">
+        <v>0</v>
+      </c>
+      <c r="T232" t="n">
+        <v>0</v>
+      </c>
+      <c r="U232" t="n">
+        <v>0</v>
+      </c>
+      <c r="V232" t="n">
+        <v>24.21900010108948</v>
+      </c>
+      <c r="W232" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="X232" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="Y232" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z232" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA232" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB232" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC232" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD232" t="inlineStr">
+        <is>
+          <t>carbon_tax_100_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE232" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260424175553_carbon_tax_100_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="B233" t="n">
+        <v>0</v>
+      </c>
+      <c r="C233" t="n">
+        <v>0</v>
+      </c>
+      <c r="D233" t="n">
+        <v>0</v>
+      </c>
+      <c r="E233" t="n">
+        <v>0</v>
+      </c>
+      <c r="F233" t="n">
+        <v>0</v>
+      </c>
+      <c r="G233" t="n">
+        <v>0</v>
+      </c>
+      <c r="H233" t="n">
+        <v>0</v>
+      </c>
+      <c r="I233" t="n">
+        <v>0</v>
+      </c>
+      <c r="J233" t="n">
+        <v>0</v>
+      </c>
+      <c r="K233" t="n">
+        <v>0</v>
+      </c>
+      <c r="L233" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="M233" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="N233" t="n">
+        <v>607492.3049917679</v>
+      </c>
+      <c r="O233" t="n">
+        <v>0</v>
+      </c>
+      <c r="P233" t="n">
+        <v>607492.3049917679</v>
+      </c>
+      <c r="Q233" t="n">
+        <v>607492.3049917654</v>
+      </c>
+      <c r="R233" t="n">
+        <v>0</v>
+      </c>
+      <c r="S233" t="n">
+        <v>0</v>
+      </c>
+      <c r="T233" t="n">
+        <v>0</v>
+      </c>
+      <c r="U233" t="n">
+        <v>0</v>
+      </c>
+      <c r="V233" t="n">
+        <v>21.00300002098083</v>
+      </c>
+      <c r="W233" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="X233" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="Y233" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z233" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA233" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB233" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC233" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD233" t="inlineStr">
+        <is>
+          <t>carbon_tax_100_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE233" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260424175949_carbon_tax_100_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="B234" t="n">
+        <v>0</v>
+      </c>
+      <c r="C234" t="n">
+        <v>0</v>
+      </c>
+      <c r="D234" t="n">
+        <v>0</v>
+      </c>
+      <c r="E234" t="n">
+        <v>0</v>
+      </c>
+      <c r="F234" t="n">
+        <v>0</v>
+      </c>
+      <c r="G234" t="n">
+        <v>0</v>
+      </c>
+      <c r="H234" t="n">
+        <v>0</v>
+      </c>
+      <c r="I234" t="n">
+        <v>0</v>
+      </c>
+      <c r="J234" t="n">
+        <v>0</v>
+      </c>
+      <c r="K234" t="n">
+        <v>0</v>
+      </c>
+      <c r="L234" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="M234" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="N234" t="n">
+        <v>607492.3049917679</v>
+      </c>
+      <c r="O234" t="n">
+        <v>0</v>
+      </c>
+      <c r="P234" t="n">
+        <v>607492.3049917679</v>
+      </c>
+      <c r="Q234" t="n">
+        <v>607492.3049917654</v>
+      </c>
+      <c r="R234" t="n">
+        <v>0</v>
+      </c>
+      <c r="S234" t="n">
+        <v>0</v>
+      </c>
+      <c r="T234" t="n">
+        <v>0</v>
+      </c>
+      <c r="U234" t="n">
+        <v>0</v>
+      </c>
+      <c r="V234" t="n">
+        <v>17.07299995422363</v>
+      </c>
+      <c r="W234" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="X234" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="Y234" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z234" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA234" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB234" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC234" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD234" t="inlineStr">
+        <is>
+          <t>carbon_tax_100_el_price_250</t>
+        </is>
+      </c>
+      <c r="AE234" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260424180321_carbon_tax_100_el_price_250</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="n">
+        <v>57115699.35527965</v>
+      </c>
+      <c r="B235" t="n">
+        <v>15828554.68961274</v>
+      </c>
+      <c r="C235" t="n">
+        <v>5951746.544758592</v>
+      </c>
+      <c r="D235" t="n">
+        <v>9950906.361202966</v>
+      </c>
+      <c r="E235" t="n">
+        <v>0</v>
+      </c>
+      <c r="F235" t="n">
+        <v>25779461.0508157</v>
+      </c>
+      <c r="G235" t="n">
+        <v>5951746.544758592</v>
+      </c>
+      <c r="H235" t="n">
+        <v>16272107.18482895</v>
+      </c>
+      <c r="I235" t="n">
+        <v>0</v>
+      </c>
+      <c r="J235" t="n">
+        <v>0</v>
+      </c>
+      <c r="K235" t="n">
+        <v>0</v>
+      </c>
+      <c r="L235" t="n">
+        <v>9112384.574876415</v>
+      </c>
+      <c r="M235" t="n">
+        <v>57115699.35527965</v>
+      </c>
+      <c r="N235" t="n">
+        <v>60756.06478760711</v>
+      </c>
+      <c r="O235" t="n">
+        <v>0</v>
+      </c>
+      <c r="P235" t="n">
+        <v>60756.06478760711</v>
+      </c>
+      <c r="Q235" t="n">
+        <v>60749.23049917652</v>
+      </c>
+      <c r="R235" t="n">
+        <v>0</v>
+      </c>
+      <c r="S235" t="n">
+        <v>0</v>
+      </c>
+      <c r="T235" t="n">
+        <v>0</v>
+      </c>
+      <c r="U235" t="n">
+        <v>6.834288431157361</v>
+      </c>
+      <c r="V235" t="n">
+        <v>18.06699991226196</v>
+      </c>
+      <c r="W235" t="n">
+        <v>57115699.3552729</v>
+      </c>
+      <c r="X235" t="n">
+        <v>57115699.35527965</v>
+      </c>
+      <c r="Y235" t="n">
+        <v>6.757676601409912e-06</v>
+      </c>
+      <c r="Z235" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA235" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB235" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC235" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD235" t="inlineStr">
+        <is>
+          <t>carbon_tax_150_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE235" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260424180657_carbon_tax_150_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="n">
+        <v>67309722.25553364</v>
+      </c>
+      <c r="B236" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C236" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="D236" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E236" t="n">
+        <v>0</v>
+      </c>
+      <c r="F236" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G236" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="H236" t="n">
+        <v>14183168.38067319</v>
+      </c>
+      <c r="I236" t="n">
+        <v>0</v>
+      </c>
+      <c r="J236" t="n">
+        <v>0</v>
+      </c>
+      <c r="K236" t="n">
+        <v>0</v>
+      </c>
+      <c r="L236" t="n">
+        <v>1085645.259932406</v>
+      </c>
+      <c r="M236" t="n">
+        <v>67309722.25553364</v>
+      </c>
+      <c r="N236" t="n">
+        <v>7245.844635991099</v>
+      </c>
+      <c r="O236" t="n">
+        <v>0</v>
+      </c>
+      <c r="P236" t="n">
+        <v>7245.844635991099</v>
+      </c>
+      <c r="Q236" t="n">
+        <v>7237.635066215916</v>
+      </c>
+      <c r="R236" t="n">
+        <v>0</v>
+      </c>
+      <c r="S236" t="n">
+        <v>0</v>
+      </c>
+      <c r="T236" t="n">
+        <v>0</v>
+      </c>
+      <c r="U236" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V236" t="n">
+        <v>25.19799995422363</v>
+      </c>
+      <c r="W236" t="n">
+        <v>67309722.25552681</v>
+      </c>
+      <c r="X236" t="n">
+        <v>67309722.25553364</v>
+      </c>
+      <c r="Y236" t="n">
+        <v>6.824731826782227e-06</v>
+      </c>
+      <c r="Z236" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA236" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB236" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC236" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD236" t="inlineStr">
+        <is>
+          <t>carbon_tax_150_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE236" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260424181045_carbon_tax_150_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="n">
+        <v>73183110.28365523</v>
+      </c>
+      <c r="B237" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C237" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="D237" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E237" t="n">
+        <v>0</v>
+      </c>
+      <c r="F237" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G237" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="H237" t="n">
+        <v>20056556.40879477</v>
+      </c>
+      <c r="I237" t="n">
+        <v>0</v>
+      </c>
+      <c r="J237" t="n">
+        <v>0</v>
+      </c>
+      <c r="K237" t="n">
+        <v>0</v>
+      </c>
+      <c r="L237" t="n">
+        <v>1085645.259932396</v>
+      </c>
+      <c r="M237" t="n">
+        <v>73183110.28365523</v>
+      </c>
+      <c r="N237" t="n">
+        <v>7245.844635991023</v>
+      </c>
+      <c r="O237" t="n">
+        <v>0</v>
+      </c>
+      <c r="P237" t="n">
+        <v>7245.844635991023</v>
+      </c>
+      <c r="Q237" t="n">
+        <v>7237.635066215884</v>
+      </c>
+      <c r="R237" t="n">
+        <v>0</v>
+      </c>
+      <c r="S237" t="n">
+        <v>0</v>
+      </c>
+      <c r="T237" t="n">
+        <v>0</v>
+      </c>
+      <c r="U237" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V237" t="n">
+        <v>19.7960000038147</v>
+      </c>
+      <c r="W237" t="n">
+        <v>73183110.28364831</v>
+      </c>
+      <c r="X237" t="n">
+        <v>73183110.28365523</v>
+      </c>
+      <c r="Y237" t="n">
+        <v>6.914138793945312e-06</v>
+      </c>
+      <c r="Z237" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA237" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB237" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC237" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD237" t="inlineStr">
+        <is>
+          <t>carbon_tax_150_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE237" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260424181451_carbon_tax_150_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="n">
+        <v>76292510.26510355</v>
+      </c>
+      <c r="B238" t="n">
+        <v>13228586.17399643</v>
+      </c>
+      <c r="C238" t="n">
+        <v>5758365.764824538</v>
+      </c>
+      <c r="D238" t="n">
+        <v>23677732.02767779</v>
+      </c>
+      <c r="E238" t="n">
+        <v>0</v>
+      </c>
+      <c r="F238" t="n">
+        <v>36906318.20167422</v>
+      </c>
+      <c r="G238" t="n">
+        <v>5758365.764824538</v>
+      </c>
+      <c r="H238" t="n">
+        <v>11914921.09995709</v>
+      </c>
+      <c r="I238" t="n">
+        <v>0</v>
+      </c>
+      <c r="J238" t="n">
+        <v>0</v>
+      </c>
+      <c r="K238" t="n">
+        <v>0</v>
+      </c>
+      <c r="L238" t="n">
+        <v>21712905.1986477</v>
+      </c>
+      <c r="M238" t="n">
+        <v>76292510.26510355</v>
+      </c>
+      <c r="N238" t="n">
+        <v>144759.1919557629</v>
+      </c>
+      <c r="O238" t="n">
+        <v>0</v>
+      </c>
+      <c r="P238" t="n">
+        <v>144759.1919557629</v>
+      </c>
+      <c r="Q238" t="n">
+        <v>144752.701324317</v>
+      </c>
+      <c r="R238" t="n">
+        <v>0</v>
+      </c>
+      <c r="S238" t="n">
+        <v>0</v>
+      </c>
+      <c r="T238" t="n">
+        <v>0</v>
+      </c>
+      <c r="U238" t="n">
+        <v>6.49063144699632</v>
+      </c>
+      <c r="V238" t="n">
+        <v>17.38699984550476</v>
+      </c>
+      <c r="W238" t="n">
+        <v>76292510.26509649</v>
+      </c>
+      <c r="X238" t="n">
+        <v>76292510.26510355</v>
+      </c>
+      <c r="Y238" t="n">
+        <v>7.063150405883789e-06</v>
+      </c>
+      <c r="Z238" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA238" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB238" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC238" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD238" t="inlineStr">
+        <is>
+          <t>carbon_tax_150_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE238" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260424181745_carbon_tax_150_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="n">
+        <v>78662142.45898528</v>
+      </c>
+      <c r="B239" t="n">
+        <v>13228586.17399643</v>
+      </c>
+      <c r="C239" t="n">
+        <v>5758365.764824538</v>
+      </c>
+      <c r="D239" t="n">
+        <v>23677732.02767779</v>
+      </c>
+      <c r="E239" t="n">
+        <v>0</v>
+      </c>
+      <c r="F239" t="n">
+        <v>36906318.20167422</v>
+      </c>
+      <c r="G239" t="n">
+        <v>5758365.764824538</v>
+      </c>
+      <c r="H239" t="n">
+        <v>14284553.29383882</v>
+      </c>
+      <c r="I239" t="n">
+        <v>0</v>
+      </c>
+      <c r="J239" t="n">
+        <v>0</v>
+      </c>
+      <c r="K239" t="n">
+        <v>0</v>
+      </c>
+      <c r="L239" t="n">
+        <v>21712905.1986477</v>
+      </c>
+      <c r="M239" t="n">
+        <v>78662142.45898528</v>
+      </c>
+      <c r="N239" t="n">
+        <v>144759.1919557629</v>
+      </c>
+      <c r="O239" t="n">
+        <v>0</v>
+      </c>
+      <c r="P239" t="n">
+        <v>144759.1919557629</v>
+      </c>
+      <c r="Q239" t="n">
+        <v>144752.701324317</v>
+      </c>
+      <c r="R239" t="n">
+        <v>0</v>
+      </c>
+      <c r="S239" t="n">
+        <v>0</v>
+      </c>
+      <c r="T239" t="n">
+        <v>0</v>
+      </c>
+      <c r="U239" t="n">
+        <v>6.49063144699632</v>
+      </c>
+      <c r="V239" t="n">
+        <v>18.2020001411438</v>
+      </c>
+      <c r="W239" t="n">
+        <v>78662142.45897821</v>
+      </c>
+      <c r="X239" t="n">
+        <v>78662142.45898528</v>
+      </c>
+      <c r="Y239" t="n">
+        <v>7.078051567077637e-06</v>
+      </c>
+      <c r="Z239" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA239" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB239" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC239" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD239" t="inlineStr">
+        <is>
+          <t>carbon_tax_150_el_price_250</t>
+        </is>
+      </c>
+      <c r="AE239" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260424182159_carbon_tax_150_el_price_250</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="n">
+        <v>60153160.88023867</v>
+      </c>
+      <c r="B240" t="n">
+        <v>15828554.68961274</v>
+      </c>
+      <c r="C240" t="n">
+        <v>5951746.544758592</v>
+      </c>
+      <c r="D240" t="n">
+        <v>9950906.361202955</v>
+      </c>
+      <c r="E240" t="n">
+        <v>0</v>
+      </c>
+      <c r="F240" t="n">
+        <v>25779461.05081569</v>
+      </c>
+      <c r="G240" t="n">
+        <v>5951746.544758592</v>
+      </c>
+      <c r="H240" t="n">
+        <v>16272107.18482895</v>
+      </c>
+      <c r="I240" t="n">
+        <v>0</v>
+      </c>
+      <c r="J240" t="n">
+        <v>0</v>
+      </c>
+      <c r="K240" t="n">
+        <v>0</v>
+      </c>
+      <c r="L240" t="n">
+        <v>12149846.09983544</v>
+      </c>
+      <c r="M240" t="n">
+        <v>60153160.88023867</v>
+      </c>
+      <c r="N240" t="n">
+        <v>60756.06478760712</v>
+      </c>
+      <c r="O240" t="n">
+        <v>0</v>
+      </c>
+      <c r="P240" t="n">
+        <v>60756.06478760712</v>
+      </c>
+      <c r="Q240" t="n">
+        <v>60749.23049917654</v>
+      </c>
+      <c r="R240" t="n">
+        <v>0</v>
+      </c>
+      <c r="S240" t="n">
+        <v>0</v>
+      </c>
+      <c r="T240" t="n">
+        <v>0</v>
+      </c>
+      <c r="U240" t="n">
+        <v>6.834288431157361</v>
+      </c>
+      <c r="V240" t="n">
+        <v>16.8510000705719</v>
+      </c>
+      <c r="W240" t="n">
+        <v>59089899.5222188</v>
+      </c>
+      <c r="X240" t="n">
+        <v>60153160.88023867</v>
+      </c>
+      <c r="Y240" t="n">
+        <v>1063261.358019873</v>
+      </c>
+      <c r="Z240" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA240" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB240" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC240" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD240" t="inlineStr">
+        <is>
+          <t>carbon_tax_200_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE240" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260424182452_carbon_tax_200_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="n">
+        <v>67671604.00884447</v>
+      </c>
+      <c r="B241" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C241" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="D241" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E241" t="n">
+        <v>0</v>
+      </c>
+      <c r="F241" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G241" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="H241" t="n">
+        <v>14183168.38067319</v>
+      </c>
+      <c r="I241" t="n">
+        <v>0</v>
+      </c>
+      <c r="J241" t="n">
+        <v>0</v>
+      </c>
+      <c r="K241" t="n">
+        <v>0</v>
+      </c>
+      <c r="L241" t="n">
+        <v>1447527.013243223</v>
+      </c>
+      <c r="M241" t="n">
+        <v>67671604.00884447</v>
+      </c>
+      <c r="N241" t="n">
+        <v>7245.844635991153</v>
+      </c>
+      <c r="O241" t="n">
+        <v>0</v>
+      </c>
+      <c r="P241" t="n">
+        <v>7245.844635991153</v>
+      </c>
+      <c r="Q241" t="n">
+        <v>7237.635066215974</v>
+      </c>
+      <c r="R241" t="n">
+        <v>0</v>
+      </c>
+      <c r="S241" t="n">
+        <v>0</v>
+      </c>
+      <c r="T241" t="n">
+        <v>0</v>
+      </c>
+      <c r="U241" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V241" t="n">
+        <v>18.7739999294281</v>
+      </c>
+      <c r="W241" t="n">
+        <v>67671604.00884447</v>
+      </c>
+      <c r="X241" t="n">
+        <v>67671604.00884447</v>
+      </c>
+      <c r="Y241" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z241" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA241" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB241" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC241" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD241" t="inlineStr">
+        <is>
+          <t>carbon_tax_200_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE241" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260424182927_carbon_tax_200_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="n">
+        <v>73544992.036966</v>
+      </c>
+      <c r="B242" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C242" t="n">
+        <v>6725637.34634771</v>
+      </c>
+      <c r="D242" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E242" t="n">
+        <v>0</v>
+      </c>
+      <c r="F242" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G242" t="n">
+        <v>6725637.34634771</v>
+      </c>
+      <c r="H242" t="n">
+        <v>20056556.40879477</v>
+      </c>
+      <c r="I242" t="n">
+        <v>0</v>
+      </c>
+      <c r="J242" t="n">
+        <v>0</v>
+      </c>
+      <c r="K242" t="n">
+        <v>0</v>
+      </c>
+      <c r="L242" t="n">
+        <v>1447527.013243163</v>
+      </c>
+      <c r="M242" t="n">
+        <v>73544992.036966</v>
+      </c>
+      <c r="N242" t="n">
+        <v>7245.844635991048</v>
+      </c>
+      <c r="O242" t="n">
+        <v>0</v>
+      </c>
+      <c r="P242" t="n">
+        <v>7245.844635991048</v>
+      </c>
+      <c r="Q242" t="n">
+        <v>7237.635066215636</v>
+      </c>
+      <c r="R242" t="n">
+        <v>0</v>
+      </c>
+      <c r="S242" t="n">
+        <v>0</v>
+      </c>
+      <c r="T242" t="n">
+        <v>0</v>
+      </c>
+      <c r="U242" t="n">
+        <v>8.209569775222587</v>
+      </c>
+      <c r="V242" t="n">
+        <v>20.72099995613098</v>
+      </c>
+      <c r="W242" t="n">
+        <v>73544992.036966</v>
+      </c>
+      <c r="X242" t="n">
+        <v>73544992.036966</v>
+      </c>
+      <c r="Y242" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z242" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA242" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB242" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC242" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD242" t="inlineStr">
+        <is>
+          <t>carbon_tax_200_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE242" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260424183224_carbon_tax_200_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="n">
+        <v>79418380.06508745</v>
+      </c>
+      <c r="B243" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C243" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="D243" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E243" t="n">
+        <v>0</v>
+      </c>
+      <c r="F243" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G243" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="H243" t="n">
+        <v>25929944.43691619</v>
+      </c>
+      <c r="I243" t="n">
+        <v>0</v>
+      </c>
+      <c r="J243" t="n">
+        <v>0</v>
+      </c>
+      <c r="K243" t="n">
+        <v>0</v>
+      </c>
+      <c r="L243" t="n">
+        <v>1447527.013243193</v>
+      </c>
+      <c r="M243" t="n">
+        <v>79418380.06508745</v>
+      </c>
+      <c r="N243" t="n">
+        <v>7245.844635991023</v>
+      </c>
+      <c r="O243" t="n">
+        <v>0</v>
+      </c>
+      <c r="P243" t="n">
+        <v>7245.844635991023</v>
+      </c>
+      <c r="Q243" t="n">
+        <v>7237.635066215884</v>
+      </c>
+      <c r="R243" t="n">
+        <v>0</v>
+      </c>
+      <c r="S243" t="n">
+        <v>0</v>
+      </c>
+      <c r="T243" t="n">
+        <v>0</v>
+      </c>
+      <c r="U243" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V243" t="n">
+        <v>19.24100017547607</v>
+      </c>
+      <c r="W243" t="n">
+        <v>79418380.06508745</v>
+      </c>
+      <c r="X243" t="n">
+        <v>79418380.06508745</v>
+      </c>
+      <c r="Y243" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z243" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA243" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB243" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC243" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD243" t="inlineStr">
+        <is>
+          <t>carbon_tax_200_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE243" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260424183726_carbon_tax_200_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="n">
+        <v>85291768.09320897</v>
+      </c>
+      <c r="B244" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C244" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="D244" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E244" t="n">
+        <v>0</v>
+      </c>
+      <c r="F244" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G244" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="H244" t="n">
+        <v>31803332.46503772</v>
+      </c>
+      <c r="I244" t="n">
+        <v>0</v>
+      </c>
+      <c r="J244" t="n">
+        <v>0</v>
+      </c>
+      <c r="K244" t="n">
+        <v>0</v>
+      </c>
+      <c r="L244" t="n">
+        <v>1447527.013243193</v>
+      </c>
+      <c r="M244" t="n">
+        <v>85291768.09320897</v>
+      </c>
+      <c r="N244" t="n">
+        <v>7245.844635991023</v>
+      </c>
+      <c r="O244" t="n">
+        <v>0</v>
+      </c>
+      <c r="P244" t="n">
+        <v>7245.844635991023</v>
+      </c>
+      <c r="Q244" t="n">
+        <v>7237.635066215884</v>
+      </c>
+      <c r="R244" t="n">
+        <v>0</v>
+      </c>
+      <c r="S244" t="n">
+        <v>0</v>
+      </c>
+      <c r="T244" t="n">
+        <v>0</v>
+      </c>
+      <c r="U244" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V244" t="n">
+        <v>19.83500003814697</v>
+      </c>
+      <c r="W244" t="n">
+        <v>85291768.09320897</v>
+      </c>
+      <c r="X244" t="n">
+        <v>85291768.09320897</v>
+      </c>
+      <c r="Y244" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z244" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA244" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB244" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC244" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD244" t="inlineStr">
+        <is>
+          <t>carbon_tax_200_el_price_250</t>
+        </is>
+      </c>
+      <c r="AE244" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260424184027_carbon_tax_200_el_price_250</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="n">
+        <v>62160097.7340337</v>
+      </c>
+      <c r="B245" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C245" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="D245" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E245" t="n">
+        <v>0</v>
+      </c>
+      <c r="F245" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G245" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="H245" t="n">
+        <v>8309780.352551687</v>
+      </c>
+      <c r="I245" t="n">
+        <v>0</v>
+      </c>
+      <c r="J245" t="n">
+        <v>0</v>
+      </c>
+      <c r="K245" t="n">
+        <v>0</v>
+      </c>
+      <c r="L245" t="n">
+        <v>1809408.766553958</v>
+      </c>
+      <c r="M245" t="n">
+        <v>62160097.7340337</v>
+      </c>
+      <c r="N245" t="n">
+        <v>7245.844635991043</v>
+      </c>
+      <c r="O245" t="n">
+        <v>0</v>
+      </c>
+      <c r="P245" t="n">
+        <v>7245.844635991043</v>
+      </c>
+      <c r="Q245" t="n">
+        <v>7237.635066215894</v>
+      </c>
+      <c r="R245" t="n">
+        <v>0</v>
+      </c>
+      <c r="S245" t="n">
+        <v>0</v>
+      </c>
+      <c r="T245" t="n">
+        <v>0</v>
+      </c>
+      <c r="U245" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V245" t="n">
+        <v>22.18599987030029</v>
+      </c>
+      <c r="W245" t="n">
+        <v>62160097.7340337</v>
+      </c>
+      <c r="X245" t="n">
+        <v>62160097.7340337</v>
+      </c>
+      <c r="Y245" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z245" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA245" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB245" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC245" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD245" t="inlineStr">
+        <is>
+          <t>carbon_tax_250_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE245" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260424184329_carbon_tax_250_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="n">
+        <v>68033485.76215513</v>
+      </c>
+      <c r="B246" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C246" t="n">
+        <v>6725637.34634771</v>
+      </c>
+      <c r="D246" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E246" t="n">
+        <v>0</v>
+      </c>
+      <c r="F246" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G246" t="n">
+        <v>6725637.34634771</v>
+      </c>
+      <c r="H246" t="n">
+        <v>14183168.3806732</v>
+      </c>
+      <c r="I246" t="n">
+        <v>0</v>
+      </c>
+      <c r="J246" t="n">
+        <v>0</v>
+      </c>
+      <c r="K246" t="n">
+        <v>0</v>
+      </c>
+      <c r="L246" t="n">
+        <v>1809408.766553886</v>
+      </c>
+      <c r="M246" t="n">
+        <v>68033485.76215513</v>
+      </c>
+      <c r="N246" t="n">
+        <v>7245.844635990788</v>
+      </c>
+      <c r="O246" t="n">
+        <v>0</v>
+      </c>
+      <c r="P246" t="n">
+        <v>7245.844635990788</v>
+      </c>
+      <c r="Q246" t="n">
+        <v>7237.635066215857</v>
+      </c>
+      <c r="R246" t="n">
+        <v>0</v>
+      </c>
+      <c r="S246" t="n">
+        <v>0</v>
+      </c>
+      <c r="T246" t="n">
+        <v>0</v>
+      </c>
+      <c r="U246" t="n">
+        <v>8.209569775222588</v>
+      </c>
+      <c r="V246" t="n">
+        <v>22.98099994659424</v>
+      </c>
+      <c r="W246" t="n">
+        <v>68033485.76215513</v>
+      </c>
+      <c r="X246" t="n">
+        <v>68033485.76215513</v>
+      </c>
+      <c r="Y246" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z246" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA246" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB246" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC246" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD246" t="inlineStr">
+        <is>
+          <t>carbon_tax_250_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE246" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260424184909_carbon_tax_250_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="n">
+        <v>73906873.79027677</v>
+      </c>
+      <c r="B247" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C247" t="n">
+        <v>6725637.34634771</v>
+      </c>
+      <c r="D247" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E247" t="n">
+        <v>0</v>
+      </c>
+      <c r="F247" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G247" t="n">
+        <v>6725637.34634771</v>
+      </c>
+      <c r="H247" t="n">
+        <v>20056556.40879477</v>
+      </c>
+      <c r="I247" t="n">
+        <v>0</v>
+      </c>
+      <c r="J247" t="n">
+        <v>0</v>
+      </c>
+      <c r="K247" t="n">
+        <v>0</v>
+      </c>
+      <c r="L247" t="n">
+        <v>1809408.766553942</v>
+      </c>
+      <c r="M247" t="n">
+        <v>73906873.79027677</v>
+      </c>
+      <c r="N247" t="n">
+        <v>7245.844635991067</v>
+      </c>
+      <c r="O247" t="n">
+        <v>0</v>
+      </c>
+      <c r="P247" t="n">
+        <v>7245.844635991067</v>
+      </c>
+      <c r="Q247" t="n">
+        <v>7237.635066215714</v>
+      </c>
+      <c r="R247" t="n">
+        <v>0</v>
+      </c>
+      <c r="S247" t="n">
+        <v>0</v>
+      </c>
+      <c r="T247" t="n">
+        <v>0</v>
+      </c>
+      <c r="U247" t="n">
+        <v>8.209569775222587</v>
+      </c>
+      <c r="V247" t="n">
+        <v>21.56599998474121</v>
+      </c>
+      <c r="W247" t="n">
+        <v>73906873.79027677</v>
+      </c>
+      <c r="X247" t="n">
+        <v>73906873.79027677</v>
+      </c>
+      <c r="Y247" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z247" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA247" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB247" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC247" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD247" t="inlineStr">
+        <is>
+          <t>carbon_tax_250_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE247" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260424185216_carbon_tax_250_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="n">
+        <v>79780261.81839819</v>
+      </c>
+      <c r="B248" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C248" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="D248" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E248" t="n">
+        <v>0</v>
+      </c>
+      <c r="F248" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G248" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="H248" t="n">
+        <v>25929944.4369162</v>
+      </c>
+      <c r="I248" t="n">
+        <v>0</v>
+      </c>
+      <c r="J248" t="n">
+        <v>0</v>
+      </c>
+      <c r="K248" t="n">
+        <v>0</v>
+      </c>
+      <c r="L248" t="n">
+        <v>1809408.766553936</v>
+      </c>
+      <c r="M248" t="n">
+        <v>79780261.81839819</v>
+      </c>
+      <c r="N248" t="n">
+        <v>7245.844635991046</v>
+      </c>
+      <c r="O248" t="n">
+        <v>0</v>
+      </c>
+      <c r="P248" t="n">
+        <v>7245.844635991046</v>
+      </c>
+      <c r="Q248" t="n">
+        <v>7237.635066215647</v>
+      </c>
+      <c r="R248" t="n">
+        <v>0</v>
+      </c>
+      <c r="S248" t="n">
+        <v>0</v>
+      </c>
+      <c r="T248" t="n">
+        <v>0</v>
+      </c>
+      <c r="U248" t="n">
+        <v>8.209569775222587</v>
+      </c>
+      <c r="V248" t="n">
+        <v>22.64000010490417</v>
+      </c>
+      <c r="W248" t="n">
+        <v>79780261.81839819</v>
+      </c>
+      <c r="X248" t="n">
+        <v>79780261.81839819</v>
+      </c>
+      <c r="Y248" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z248" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA248" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB248" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC248" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD248" t="inlineStr">
+        <is>
+          <t>carbon_tax_250_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE248" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260424185520_carbon_tax_250_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="n">
+        <v>85653649.84651972</v>
+      </c>
+      <c r="B249" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C249" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="D249" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E249" t="n">
+        <v>0</v>
+      </c>
+      <c r="F249" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G249" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="H249" t="n">
+        <v>31803332.46503772</v>
+      </c>
+      <c r="I249" t="n">
+        <v>0</v>
+      </c>
+      <c r="J249" t="n">
+        <v>0</v>
+      </c>
+      <c r="K249" t="n">
+        <v>0</v>
+      </c>
+      <c r="L249" t="n">
+        <v>1809408.766553953</v>
+      </c>
+      <c r="M249" t="n">
+        <v>85653649.84651972</v>
+      </c>
+      <c r="N249" t="n">
+        <v>7245.844635991023</v>
+      </c>
+      <c r="O249" t="n">
+        <v>0</v>
+      </c>
+      <c r="P249" t="n">
+        <v>7245.844635991023</v>
+      </c>
+      <c r="Q249" t="n">
+        <v>7237.635066215884</v>
+      </c>
+      <c r="R249" t="n">
+        <v>0</v>
+      </c>
+      <c r="S249" t="n">
+        <v>0</v>
+      </c>
+      <c r="T249" t="n">
+        <v>0</v>
+      </c>
+      <c r="U249" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V249" t="n">
+        <v>22.84599995613098</v>
+      </c>
+      <c r="W249" t="n">
+        <v>85653649.84651972</v>
+      </c>
+      <c r="X249" t="n">
+        <v>85653649.84651972</v>
+      </c>
+      <c r="Y249" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z249" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA249" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB249" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC249" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD249" t="inlineStr">
+        <is>
+          <t>carbon_tax_250_el_price_250</t>
+        </is>
+      </c>
+      <c r="AE249" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260424185822_carbon_tax_250_el_price_250</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="n">
+        <v>62521979.48734454</v>
+      </c>
+      <c r="B250" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C250" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="D250" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E250" t="n">
+        <v>0</v>
+      </c>
+      <c r="F250" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G250" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="H250" t="n">
+        <v>8309780.352551686</v>
+      </c>
+      <c r="I250" t="n">
+        <v>0</v>
+      </c>
+      <c r="J250" t="n">
+        <v>0</v>
+      </c>
+      <c r="K250" t="n">
+        <v>0</v>
+      </c>
+      <c r="L250" t="n">
+        <v>2171290.519864808</v>
+      </c>
+      <c r="M250" t="n">
+        <v>62521979.48734454</v>
+      </c>
+      <c r="N250" t="n">
+        <v>7245.844635991087</v>
+      </c>
+      <c r="O250" t="n">
+        <v>0</v>
+      </c>
+      <c r="P250" t="n">
+        <v>7245.844635991087</v>
+      </c>
+      <c r="Q250" t="n">
+        <v>7237.635066215911</v>
+      </c>
+      <c r="R250" t="n">
+        <v>0</v>
+      </c>
+      <c r="S250" t="n">
+        <v>0</v>
+      </c>
+      <c r="T250" t="n">
+        <v>0</v>
+      </c>
+      <c r="U250" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V250" t="n">
+        <v>20.95899987220764</v>
+      </c>
+      <c r="W250" t="n">
+        <v>62521979.48732942</v>
+      </c>
+      <c r="X250" t="n">
+        <v>62521979.48734454</v>
+      </c>
+      <c r="Y250" t="n">
+        <v>1.511722803115845e-05</v>
+      </c>
+      <c r="Z250" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA250" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB250" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC250" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD250" t="inlineStr">
+        <is>
+          <t>carbon_tax_300_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE250" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260424190434_carbon_tax_300_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="n">
+        <v>68395367.51546599</v>
+      </c>
+      <c r="B251" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C251" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="D251" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E251" t="n">
+        <v>0</v>
+      </c>
+      <c r="F251" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G251" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="H251" t="n">
+        <v>14183168.38067319</v>
+      </c>
+      <c r="I251" t="n">
+        <v>0</v>
+      </c>
+      <c r="J251" t="n">
+        <v>0</v>
+      </c>
+      <c r="K251" t="n">
+        <v>0</v>
+      </c>
+      <c r="L251" t="n">
+        <v>2171290.519864745</v>
+      </c>
+      <c r="M251" t="n">
+        <v>68395367.51546599</v>
+      </c>
+      <c r="N251" t="n">
+        <v>7245.844635990953</v>
+      </c>
+      <c r="O251" t="n">
+        <v>0</v>
+      </c>
+      <c r="P251" t="n">
+        <v>7245.844635990953</v>
+      </c>
+      <c r="Q251" t="n">
+        <v>7237.63506621585</v>
+      </c>
+      <c r="R251" t="n">
+        <v>0</v>
+      </c>
+      <c r="S251" t="n">
+        <v>0</v>
+      </c>
+      <c r="T251" t="n">
+        <v>0</v>
+      </c>
+      <c r="U251" t="n">
+        <v>8.209569775222587</v>
+      </c>
+      <c r="V251" t="n">
+        <v>23.85699987411499</v>
+      </c>
+      <c r="W251" t="n">
+        <v>68395367.51545092</v>
+      </c>
+      <c r="X251" t="n">
+        <v>68395367.51546599</v>
+      </c>
+      <c r="Y251" t="n">
+        <v>1.506507396697998e-05</v>
+      </c>
+      <c r="Z251" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA251" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB251" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC251" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD251" t="inlineStr">
+        <is>
+          <t>carbon_tax_300_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE251" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260424190732_carbon_tax_300_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="n">
+        <v>74268755.54358758</v>
+      </c>
+      <c r="B252" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C252" t="n">
+        <v>6725637.34634771</v>
+      </c>
+      <c r="D252" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E252" t="n">
+        <v>0</v>
+      </c>
+      <c r="F252" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G252" t="n">
+        <v>6725637.34634771</v>
+      </c>
+      <c r="H252" t="n">
+        <v>20056556.40879477</v>
+      </c>
+      <c r="I252" t="n">
+        <v>0</v>
+      </c>
+      <c r="J252" t="n">
+        <v>0</v>
+      </c>
+      <c r="K252" t="n">
+        <v>0</v>
+      </c>
+      <c r="L252" t="n">
+        <v>2171290.51986475</v>
+      </c>
+      <c r="M252" t="n">
+        <v>74268755.54358758</v>
+      </c>
+      <c r="N252" t="n">
+        <v>7245.844635991049</v>
+      </c>
+      <c r="O252" t="n">
+        <v>0</v>
+      </c>
+      <c r="P252" t="n">
+        <v>7245.844635991049</v>
+      </c>
+      <c r="Q252" t="n">
+        <v>7237.635066215772</v>
+      </c>
+      <c r="R252" t="n">
+        <v>0</v>
+      </c>
+      <c r="S252" t="n">
+        <v>0</v>
+      </c>
+      <c r="T252" t="n">
+        <v>0</v>
+      </c>
+      <c r="U252" t="n">
+        <v>8.209569775222585</v>
+      </c>
+      <c r="V252" t="n">
+        <v>23.89100003242493</v>
+      </c>
+      <c r="W252" t="n">
+        <v>74268755.54357257</v>
+      </c>
+      <c r="X252" t="n">
+        <v>74268755.54358758</v>
+      </c>
+      <c r="Y252" t="n">
+        <v>1.500546932220459e-05</v>
+      </c>
+      <c r="Z252" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA252" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB252" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC252" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD252" t="inlineStr">
+        <is>
+          <t>carbon_tax_300_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE252" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260424191035_carbon_tax_300_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="n">
+        <v>80142143.57170908</v>
+      </c>
+      <c r="B253" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C253" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="D253" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E253" t="n">
+        <v>0</v>
+      </c>
+      <c r="F253" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G253" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="H253" t="n">
+        <v>25929944.4369162</v>
+      </c>
+      <c r="I253" t="n">
+        <v>0</v>
+      </c>
+      <c r="J253" t="n">
+        <v>0</v>
+      </c>
+      <c r="K253" t="n">
+        <v>0</v>
+      </c>
+      <c r="L253" t="n">
+        <v>2171290.519864827</v>
+      </c>
+      <c r="M253" t="n">
+        <v>80142143.57170908</v>
+      </c>
+      <c r="N253" t="n">
+        <v>7245.844635991149</v>
+      </c>
+      <c r="O253" t="n">
+        <v>0</v>
+      </c>
+      <c r="P253" t="n">
+        <v>7245.844635991149</v>
+      </c>
+      <c r="Q253" t="n">
+        <v>7237.635066215967</v>
+      </c>
+      <c r="R253" t="n">
+        <v>0</v>
+      </c>
+      <c r="S253" t="n">
+        <v>0</v>
+      </c>
+      <c r="T253" t="n">
+        <v>0</v>
+      </c>
+      <c r="U253" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V253" t="n">
+        <v>25.10199999809265</v>
+      </c>
+      <c r="W253" t="n">
+        <v>80142143.57169431</v>
+      </c>
+      <c r="X253" t="n">
+        <v>80142143.57170908</v>
+      </c>
+      <c r="Y253" t="n">
+        <v>1.476705074310303e-05</v>
+      </c>
+      <c r="Z253" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA253" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB253" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC253" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD253" t="inlineStr">
+        <is>
+          <t>carbon_tax_300_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE253" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260424191341_carbon_tax_300_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="n">
+        <v>86015531.59983046</v>
+      </c>
+      <c r="B254" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C254" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="D254" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E254" t="n">
+        <v>0</v>
+      </c>
+      <c r="F254" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G254" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="H254" t="n">
+        <v>31803332.46503773</v>
+      </c>
+      <c r="I254" t="n">
+        <v>0</v>
+      </c>
+      <c r="J254" t="n">
+        <v>0</v>
+      </c>
+      <c r="K254" t="n">
+        <v>0</v>
+      </c>
+      <c r="L254" t="n">
+        <v>2171290.519864698</v>
+      </c>
+      <c r="M254" t="n">
+        <v>86015531.59983046</v>
+      </c>
+      <c r="N254" t="n">
+        <v>7245.844635991034</v>
+      </c>
+      <c r="O254" t="n">
+        <v>0</v>
+      </c>
+      <c r="P254" t="n">
+        <v>7245.844635991034</v>
+      </c>
+      <c r="Q254" t="n">
+        <v>7237.635066215644</v>
+      </c>
+      <c r="R254" t="n">
+        <v>0</v>
+      </c>
+      <c r="S254" t="n">
+        <v>0</v>
+      </c>
+      <c r="T254" t="n">
+        <v>0</v>
+      </c>
+      <c r="U254" t="n">
+        <v>8.209569775222587</v>
+      </c>
+      <c r="V254" t="n">
+        <v>25.43900012969971</v>
+      </c>
+      <c r="W254" t="n">
+        <v>86015531.59981586</v>
+      </c>
+      <c r="X254" t="n">
+        <v>86015531.59983046</v>
+      </c>
+      <c r="Y254" t="n">
+        <v>1.46031379699707e-05</v>
+      </c>
+      <c r="Z254" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA254" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB254" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC254" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD254" t="inlineStr">
+        <is>
+          <t>carbon_tax_300_el_price_250</t>
+        </is>
+      </c>
+      <c r="AE254" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260424192043_carbon_tax_300_el_price_250</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
results with updated HP cost
</commit_message>
<xml_diff>
--- a/dataCaseStudy_Cement/raw_results/tech_selection/Summary.xlsx
+++ b/dataCaseStudy_Cement/raw_results/tech_selection/Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE304"/>
+  <dimension ref="A1:AE329"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31791,6 +31791,2581 @@
       <c r="AE304" t="inlineStr">
         <is>
           <t>dataCaseStudy_Cement\raw_results\tech_selection\20260428124831_carbon_tax_300_el_price_250</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="n">
+        <v>55807148.464256</v>
+      </c>
+      <c r="B305" t="n">
+        <v>14404244.23429233</v>
+      </c>
+      <c r="C305" t="n">
+        <v>5951746.544758592</v>
+      </c>
+      <c r="D305" t="n">
+        <v>13104127.45045842</v>
+      </c>
+      <c r="E305" t="n">
+        <v>0</v>
+      </c>
+      <c r="F305" t="n">
+        <v>27508371.68475074</v>
+      </c>
+      <c r="G305" t="n">
+        <v>5951746.544758592</v>
+      </c>
+      <c r="H305" t="n">
+        <v>16272107.18482895</v>
+      </c>
+      <c r="I305" t="n">
+        <v>0</v>
+      </c>
+      <c r="J305" t="n">
+        <v>0</v>
+      </c>
+      <c r="K305" t="n">
+        <v>0</v>
+      </c>
+      <c r="L305" t="n">
+        <v>6074923.049917719</v>
+      </c>
+      <c r="M305" t="n">
+        <v>55807148.464256</v>
+      </c>
+      <c r="N305" t="n">
+        <v>60756.06478760712</v>
+      </c>
+      <c r="O305" t="n">
+        <v>0</v>
+      </c>
+      <c r="P305" t="n">
+        <v>60756.06478760712</v>
+      </c>
+      <c r="Q305" t="n">
+        <v>60749.23049917654</v>
+      </c>
+      <c r="R305" t="n">
+        <v>0</v>
+      </c>
+      <c r="S305" t="n">
+        <v>0</v>
+      </c>
+      <c r="T305" t="n">
+        <v>0</v>
+      </c>
+      <c r="U305" t="n">
+        <v>6.834288431157361</v>
+      </c>
+      <c r="V305" t="n">
+        <v>21.07200002670288</v>
+      </c>
+      <c r="W305" t="n">
+        <v>54691245.19128505</v>
+      </c>
+      <c r="X305" t="n">
+        <v>55807148.464256</v>
+      </c>
+      <c r="Y305" t="n">
+        <v>1115903.272970952</v>
+      </c>
+      <c r="Z305" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA305" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB305" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC305" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD305" t="inlineStr">
+        <is>
+          <t>carbon_tax_100_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE305" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260806111827_carbon_tax_100_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="B306" t="n">
+        <v>0</v>
+      </c>
+      <c r="C306" t="n">
+        <v>0</v>
+      </c>
+      <c r="D306" t="n">
+        <v>0</v>
+      </c>
+      <c r="E306" t="n">
+        <v>0</v>
+      </c>
+      <c r="F306" t="n">
+        <v>0</v>
+      </c>
+      <c r="G306" t="n">
+        <v>0</v>
+      </c>
+      <c r="H306" t="n">
+        <v>0</v>
+      </c>
+      <c r="I306" t="n">
+        <v>0</v>
+      </c>
+      <c r="J306" t="n">
+        <v>0</v>
+      </c>
+      <c r="K306" t="n">
+        <v>0</v>
+      </c>
+      <c r="L306" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="M306" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="N306" t="n">
+        <v>607492.3049917679</v>
+      </c>
+      <c r="O306" t="n">
+        <v>0</v>
+      </c>
+      <c r="P306" t="n">
+        <v>607492.3049917679</v>
+      </c>
+      <c r="Q306" t="n">
+        <v>607492.3049917654</v>
+      </c>
+      <c r="R306" t="n">
+        <v>0</v>
+      </c>
+      <c r="S306" t="n">
+        <v>0</v>
+      </c>
+      <c r="T306" t="n">
+        <v>0</v>
+      </c>
+      <c r="U306" t="n">
+        <v>0</v>
+      </c>
+      <c r="V306" t="n">
+        <v>29.81399989128113</v>
+      </c>
+      <c r="W306" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="X306" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="Y306" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z306" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA306" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB306" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC306" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD306" t="inlineStr">
+        <is>
+          <t>carbon_tax_100_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE306" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260806112215_carbon_tax_100_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="B307" t="n">
+        <v>0</v>
+      </c>
+      <c r="C307" t="n">
+        <v>0</v>
+      </c>
+      <c r="D307" t="n">
+        <v>0</v>
+      </c>
+      <c r="E307" t="n">
+        <v>0</v>
+      </c>
+      <c r="F307" t="n">
+        <v>0</v>
+      </c>
+      <c r="G307" t="n">
+        <v>0</v>
+      </c>
+      <c r="H307" t="n">
+        <v>0</v>
+      </c>
+      <c r="I307" t="n">
+        <v>0</v>
+      </c>
+      <c r="J307" t="n">
+        <v>0</v>
+      </c>
+      <c r="K307" t="n">
+        <v>0</v>
+      </c>
+      <c r="L307" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="M307" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="N307" t="n">
+        <v>607492.3049917679</v>
+      </c>
+      <c r="O307" t="n">
+        <v>0</v>
+      </c>
+      <c r="P307" t="n">
+        <v>607492.3049917679</v>
+      </c>
+      <c r="Q307" t="n">
+        <v>607492.3049917654</v>
+      </c>
+      <c r="R307" t="n">
+        <v>0</v>
+      </c>
+      <c r="S307" t="n">
+        <v>0</v>
+      </c>
+      <c r="T307" t="n">
+        <v>0</v>
+      </c>
+      <c r="U307" t="n">
+        <v>0</v>
+      </c>
+      <c r="V307" t="n">
+        <v>25.39100003242493</v>
+      </c>
+      <c r="W307" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="X307" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="Y307" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z307" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA307" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB307" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC307" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD307" t="inlineStr">
+        <is>
+          <t>carbon_tax_100_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE307" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260806112605_carbon_tax_100_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="B308" t="n">
+        <v>0</v>
+      </c>
+      <c r="C308" t="n">
+        <v>0</v>
+      </c>
+      <c r="D308" t="n">
+        <v>0</v>
+      </c>
+      <c r="E308" t="n">
+        <v>0</v>
+      </c>
+      <c r="F308" t="n">
+        <v>0</v>
+      </c>
+      <c r="G308" t="n">
+        <v>0</v>
+      </c>
+      <c r="H308" t="n">
+        <v>0</v>
+      </c>
+      <c r="I308" t="n">
+        <v>0</v>
+      </c>
+      <c r="J308" t="n">
+        <v>0</v>
+      </c>
+      <c r="K308" t="n">
+        <v>0</v>
+      </c>
+      <c r="L308" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="M308" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="N308" t="n">
+        <v>607492.3049917679</v>
+      </c>
+      <c r="O308" t="n">
+        <v>0</v>
+      </c>
+      <c r="P308" t="n">
+        <v>607492.3049917679</v>
+      </c>
+      <c r="Q308" t="n">
+        <v>607492.3049917654</v>
+      </c>
+      <c r="R308" t="n">
+        <v>0</v>
+      </c>
+      <c r="S308" t="n">
+        <v>0</v>
+      </c>
+      <c r="T308" t="n">
+        <v>0</v>
+      </c>
+      <c r="U308" t="n">
+        <v>0</v>
+      </c>
+      <c r="V308" t="n">
+        <v>24.74499988555908</v>
+      </c>
+      <c r="W308" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="X308" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="Y308" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z308" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA308" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB308" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC308" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD308" t="inlineStr">
+        <is>
+          <t>carbon_tax_100_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE308" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260806113012_carbon_tax_100_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="B309" t="n">
+        <v>0</v>
+      </c>
+      <c r="C309" t="n">
+        <v>0</v>
+      </c>
+      <c r="D309" t="n">
+        <v>0</v>
+      </c>
+      <c r="E309" t="n">
+        <v>0</v>
+      </c>
+      <c r="F309" t="n">
+        <v>0</v>
+      </c>
+      <c r="G309" t="n">
+        <v>0</v>
+      </c>
+      <c r="H309" t="n">
+        <v>0</v>
+      </c>
+      <c r="I309" t="n">
+        <v>0</v>
+      </c>
+      <c r="J309" t="n">
+        <v>0</v>
+      </c>
+      <c r="K309" t="n">
+        <v>0</v>
+      </c>
+      <c r="L309" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="M309" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="N309" t="n">
+        <v>607492.3049917679</v>
+      </c>
+      <c r="O309" t="n">
+        <v>0</v>
+      </c>
+      <c r="P309" t="n">
+        <v>607492.3049917679</v>
+      </c>
+      <c r="Q309" t="n">
+        <v>607492.3049917654</v>
+      </c>
+      <c r="R309" t="n">
+        <v>0</v>
+      </c>
+      <c r="S309" t="n">
+        <v>0</v>
+      </c>
+      <c r="T309" t="n">
+        <v>0</v>
+      </c>
+      <c r="U309" t="n">
+        <v>0</v>
+      </c>
+      <c r="V309" t="n">
+        <v>17.95499992370605</v>
+      </c>
+      <c r="W309" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="X309" t="n">
+        <v>60749230.49917586</v>
+      </c>
+      <c r="Y309" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z309" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA309" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB309" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC309" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD309" t="inlineStr">
+        <is>
+          <t>carbon_tax_100_el_price_250</t>
+        </is>
+      </c>
+      <c r="AE309" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260806113405_carbon_tax_100_el_price_250</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="n">
+        <v>58844609.9892147</v>
+      </c>
+      <c r="B310" t="n">
+        <v>14404244.23429233</v>
+      </c>
+      <c r="C310" t="n">
+        <v>5951746.544758592</v>
+      </c>
+      <c r="D310" t="n">
+        <v>13104127.45045842</v>
+      </c>
+      <c r="E310" t="n">
+        <v>0</v>
+      </c>
+      <c r="F310" t="n">
+        <v>27508371.68475074</v>
+      </c>
+      <c r="G310" t="n">
+        <v>5951746.544758592</v>
+      </c>
+      <c r="H310" t="n">
+        <v>16272107.18482895</v>
+      </c>
+      <c r="I310" t="n">
+        <v>0</v>
+      </c>
+      <c r="J310" t="n">
+        <v>0</v>
+      </c>
+      <c r="K310" t="n">
+        <v>0</v>
+      </c>
+      <c r="L310" t="n">
+        <v>9112384.574876415</v>
+      </c>
+      <c r="M310" t="n">
+        <v>58844609.9892147</v>
+      </c>
+      <c r="N310" t="n">
+        <v>60756.06478760712</v>
+      </c>
+      <c r="O310" t="n">
+        <v>0</v>
+      </c>
+      <c r="P310" t="n">
+        <v>60756.06478760712</v>
+      </c>
+      <c r="Q310" t="n">
+        <v>60749.23049917654</v>
+      </c>
+      <c r="R310" t="n">
+        <v>0</v>
+      </c>
+      <c r="S310" t="n">
+        <v>0</v>
+      </c>
+      <c r="T310" t="n">
+        <v>0</v>
+      </c>
+      <c r="U310" t="n">
+        <v>6.834288431157361</v>
+      </c>
+      <c r="V310" t="n">
+        <v>23.60599994659424</v>
+      </c>
+      <c r="W310" t="n">
+        <v>58844609.9892079</v>
+      </c>
+      <c r="X310" t="n">
+        <v>58844609.9892147</v>
+      </c>
+      <c r="Y310" t="n">
+        <v>6.794929504394531e-06</v>
+      </c>
+      <c r="Z310" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA310" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB310" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC310" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD310" t="inlineStr">
+        <is>
+          <t>carbon_tax_150_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE310" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260806113752_carbon_tax_150_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="n">
+        <v>67309722.25553359</v>
+      </c>
+      <c r="B311" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C311" t="n">
+        <v>6725637.346347711</v>
+      </c>
+      <c r="D311" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E311" t="n">
+        <v>0</v>
+      </c>
+      <c r="F311" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G311" t="n">
+        <v>6725637.346347711</v>
+      </c>
+      <c r="H311" t="n">
+        <v>14183168.38067319</v>
+      </c>
+      <c r="I311" t="n">
+        <v>0</v>
+      </c>
+      <c r="J311" t="n">
+        <v>0</v>
+      </c>
+      <c r="K311" t="n">
+        <v>0</v>
+      </c>
+      <c r="L311" t="n">
+        <v>1085645.259932343</v>
+      </c>
+      <c r="M311" t="n">
+        <v>67309722.25553359</v>
+      </c>
+      <c r="N311" t="n">
+        <v>7245.84463599104</v>
+      </c>
+      <c r="O311" t="n">
+        <v>0</v>
+      </c>
+      <c r="P311" t="n">
+        <v>7245.84463599104</v>
+      </c>
+      <c r="Q311" t="n">
+        <v>7237.635066215611</v>
+      </c>
+      <c r="R311" t="n">
+        <v>0</v>
+      </c>
+      <c r="S311" t="n">
+        <v>0</v>
+      </c>
+      <c r="T311" t="n">
+        <v>0</v>
+      </c>
+      <c r="U311" t="n">
+        <v>8.209569775222587</v>
+      </c>
+      <c r="V311" t="n">
+        <v>18.23799991607666</v>
+      </c>
+      <c r="W311" t="n">
+        <v>67309722.25552669</v>
+      </c>
+      <c r="X311" t="n">
+        <v>67309722.25553359</v>
+      </c>
+      <c r="Y311" t="n">
+        <v>6.899237632751465e-06</v>
+      </c>
+      <c r="Z311" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA311" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB311" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC311" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD311" t="inlineStr">
+        <is>
+          <t>carbon_tax_150_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE311" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260806114157_carbon_tax_150_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="n">
+        <v>73183110.28365523</v>
+      </c>
+      <c r="B312" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C312" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="D312" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E312" t="n">
+        <v>0</v>
+      </c>
+      <c r="F312" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G312" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="H312" t="n">
+        <v>20056556.40879477</v>
+      </c>
+      <c r="I312" t="n">
+        <v>0</v>
+      </c>
+      <c r="J312" t="n">
+        <v>0</v>
+      </c>
+      <c r="K312" t="n">
+        <v>0</v>
+      </c>
+      <c r="L312" t="n">
+        <v>1085645.259932396</v>
+      </c>
+      <c r="M312" t="n">
+        <v>73183110.28365523</v>
+      </c>
+      <c r="N312" t="n">
+        <v>7245.844635991023</v>
+      </c>
+      <c r="O312" t="n">
+        <v>0</v>
+      </c>
+      <c r="P312" t="n">
+        <v>7245.844635991023</v>
+      </c>
+      <c r="Q312" t="n">
+        <v>7237.635066215884</v>
+      </c>
+      <c r="R312" t="n">
+        <v>0</v>
+      </c>
+      <c r="S312" t="n">
+        <v>0</v>
+      </c>
+      <c r="T312" t="n">
+        <v>0</v>
+      </c>
+      <c r="U312" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V312" t="n">
+        <v>16.63900017738342</v>
+      </c>
+      <c r="W312" t="n">
+        <v>73183110.28364833</v>
+      </c>
+      <c r="X312" t="n">
+        <v>73183110.28365523</v>
+      </c>
+      <c r="Y312" t="n">
+        <v>6.899237632751465e-06</v>
+      </c>
+      <c r="Z312" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA312" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB312" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC312" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD312" t="inlineStr">
+        <is>
+          <t>carbon_tax_150_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE312" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260806114608_carbon_tax_150_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="n">
+        <v>76292510.26510355</v>
+      </c>
+      <c r="B313" t="n">
+        <v>13228586.17399643</v>
+      </c>
+      <c r="C313" t="n">
+        <v>5758365.764824538</v>
+      </c>
+      <c r="D313" t="n">
+        <v>23677732.02767779</v>
+      </c>
+      <c r="E313" t="n">
+        <v>0</v>
+      </c>
+      <c r="F313" t="n">
+        <v>36906318.20167422</v>
+      </c>
+      <c r="G313" t="n">
+        <v>5758365.764824538</v>
+      </c>
+      <c r="H313" t="n">
+        <v>11914921.09995709</v>
+      </c>
+      <c r="I313" t="n">
+        <v>0</v>
+      </c>
+      <c r="J313" t="n">
+        <v>0</v>
+      </c>
+      <c r="K313" t="n">
+        <v>0</v>
+      </c>
+      <c r="L313" t="n">
+        <v>21712905.1986477</v>
+      </c>
+      <c r="M313" t="n">
+        <v>76292510.26510355</v>
+      </c>
+      <c r="N313" t="n">
+        <v>144759.1919557629</v>
+      </c>
+      <c r="O313" t="n">
+        <v>0</v>
+      </c>
+      <c r="P313" t="n">
+        <v>144759.1919557629</v>
+      </c>
+      <c r="Q313" t="n">
+        <v>144752.701324317</v>
+      </c>
+      <c r="R313" t="n">
+        <v>0</v>
+      </c>
+      <c r="S313" t="n">
+        <v>0</v>
+      </c>
+      <c r="T313" t="n">
+        <v>0</v>
+      </c>
+      <c r="U313" t="n">
+        <v>6.49063144699632</v>
+      </c>
+      <c r="V313" t="n">
+        <v>16.89599990844727</v>
+      </c>
+      <c r="W313" t="n">
+        <v>76292510.26509649</v>
+      </c>
+      <c r="X313" t="n">
+        <v>76292510.26510355</v>
+      </c>
+      <c r="Y313" t="n">
+        <v>7.063150405883789e-06</v>
+      </c>
+      <c r="Z313" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA313" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB313" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC313" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD313" t="inlineStr">
+        <is>
+          <t>carbon_tax_150_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE313" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260806114900_carbon_tax_150_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="n">
+        <v>78662142.45898528</v>
+      </c>
+      <c r="B314" t="n">
+        <v>13228586.17399643</v>
+      </c>
+      <c r="C314" t="n">
+        <v>5758365.764824538</v>
+      </c>
+      <c r="D314" t="n">
+        <v>23677732.02767779</v>
+      </c>
+      <c r="E314" t="n">
+        <v>0</v>
+      </c>
+      <c r="F314" t="n">
+        <v>36906318.20167422</v>
+      </c>
+      <c r="G314" t="n">
+        <v>5758365.764824538</v>
+      </c>
+      <c r="H314" t="n">
+        <v>14284553.29383882</v>
+      </c>
+      <c r="I314" t="n">
+        <v>0</v>
+      </c>
+      <c r="J314" t="n">
+        <v>0</v>
+      </c>
+      <c r="K314" t="n">
+        <v>0</v>
+      </c>
+      <c r="L314" t="n">
+        <v>21712905.1986477</v>
+      </c>
+      <c r="M314" t="n">
+        <v>78662142.45898528</v>
+      </c>
+      <c r="N314" t="n">
+        <v>144759.1919557629</v>
+      </c>
+      <c r="O314" t="n">
+        <v>0</v>
+      </c>
+      <c r="P314" t="n">
+        <v>144759.1919557629</v>
+      </c>
+      <c r="Q314" t="n">
+        <v>144752.701324317</v>
+      </c>
+      <c r="R314" t="n">
+        <v>0</v>
+      </c>
+      <c r="S314" t="n">
+        <v>0</v>
+      </c>
+      <c r="T314" t="n">
+        <v>0</v>
+      </c>
+      <c r="U314" t="n">
+        <v>6.49063144699632</v>
+      </c>
+      <c r="V314" t="n">
+        <v>17.71300005912781</v>
+      </c>
+      <c r="W314" t="n">
+        <v>78662142.45897821</v>
+      </c>
+      <c r="X314" t="n">
+        <v>78662142.45898528</v>
+      </c>
+      <c r="Y314" t="n">
+        <v>7.078051567077637e-06</v>
+      </c>
+      <c r="Z314" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA314" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB314" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC314" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD314" t="inlineStr">
+        <is>
+          <t>carbon_tax_150_el_price_250</t>
+        </is>
+      </c>
+      <c r="AE314" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260806115325_carbon_tax_150_el_price_250</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="n">
+        <v>61798215.98072296</v>
+      </c>
+      <c r="B315" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C315" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="D315" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E315" t="n">
+        <v>0</v>
+      </c>
+      <c r="F315" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G315" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="H315" t="n">
+        <v>8309780.352551687</v>
+      </c>
+      <c r="I315" t="n">
+        <v>0</v>
+      </c>
+      <c r="J315" t="n">
+        <v>0</v>
+      </c>
+      <c r="K315" t="n">
+        <v>0</v>
+      </c>
+      <c r="L315" t="n">
+        <v>1447527.013243216</v>
+      </c>
+      <c r="M315" t="n">
+        <v>61798215.98072296</v>
+      </c>
+      <c r="N315" t="n">
+        <v>7245.844635991121</v>
+      </c>
+      <c r="O315" t="n">
+        <v>0</v>
+      </c>
+      <c r="P315" t="n">
+        <v>7245.844635991121</v>
+      </c>
+      <c r="Q315" t="n">
+        <v>7237.635066215956</v>
+      </c>
+      <c r="R315" t="n">
+        <v>0</v>
+      </c>
+      <c r="S315" t="n">
+        <v>0</v>
+      </c>
+      <c r="T315" t="n">
+        <v>0</v>
+      </c>
+      <c r="U315" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V315" t="n">
+        <v>16.83400011062622</v>
+      </c>
+      <c r="W315" t="n">
+        <v>61798215.98072296</v>
+      </c>
+      <c r="X315" t="n">
+        <v>61798215.98072296</v>
+      </c>
+      <c r="Y315" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z315" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA315" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB315" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC315" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD315" t="inlineStr">
+        <is>
+          <t>carbon_tax_200_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE315" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260806115618_carbon_tax_200_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="n">
+        <v>67671604.00884444</v>
+      </c>
+      <c r="B316" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C316" t="n">
+        <v>6725637.34634771</v>
+      </c>
+      <c r="D316" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E316" t="n">
+        <v>0</v>
+      </c>
+      <c r="F316" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G316" t="n">
+        <v>6725637.34634771</v>
+      </c>
+      <c r="H316" t="n">
+        <v>14183168.38067319</v>
+      </c>
+      <c r="I316" t="n">
+        <v>0</v>
+      </c>
+      <c r="J316" t="n">
+        <v>0</v>
+      </c>
+      <c r="K316" t="n">
+        <v>0</v>
+      </c>
+      <c r="L316" t="n">
+        <v>1447527.013243186</v>
+      </c>
+      <c r="M316" t="n">
+        <v>67671604.00884444</v>
+      </c>
+      <c r="N316" t="n">
+        <v>7245.844635991081</v>
+      </c>
+      <c r="O316" t="n">
+        <v>0</v>
+      </c>
+      <c r="P316" t="n">
+        <v>7245.844635991081</v>
+      </c>
+      <c r="Q316" t="n">
+        <v>7237.635066215728</v>
+      </c>
+      <c r="R316" t="n">
+        <v>0</v>
+      </c>
+      <c r="S316" t="n">
+        <v>0</v>
+      </c>
+      <c r="T316" t="n">
+        <v>0</v>
+      </c>
+      <c r="U316" t="n">
+        <v>8.209569775222587</v>
+      </c>
+      <c r="V316" t="n">
+        <v>17.52300000190735</v>
+      </c>
+      <c r="W316" t="n">
+        <v>67671604.00884444</v>
+      </c>
+      <c r="X316" t="n">
+        <v>67671604.00884444</v>
+      </c>
+      <c r="Y316" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z316" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA316" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB316" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC316" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD316" t="inlineStr">
+        <is>
+          <t>carbon_tax_200_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE316" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260806120113_carbon_tax_200_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="n">
+        <v>73544992.036966</v>
+      </c>
+      <c r="B317" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C317" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="D317" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E317" t="n">
+        <v>0</v>
+      </c>
+      <c r="F317" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G317" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="H317" t="n">
+        <v>20056556.40879477</v>
+      </c>
+      <c r="I317" t="n">
+        <v>0</v>
+      </c>
+      <c r="J317" t="n">
+        <v>0</v>
+      </c>
+      <c r="K317" t="n">
+        <v>0</v>
+      </c>
+      <c r="L317" t="n">
+        <v>1447527.013243166</v>
+      </c>
+      <c r="M317" t="n">
+        <v>73544992.036966</v>
+      </c>
+      <c r="N317" t="n">
+        <v>7245.844635991053</v>
+      </c>
+      <c r="O317" t="n">
+        <v>0</v>
+      </c>
+      <c r="P317" t="n">
+        <v>7245.844635991053</v>
+      </c>
+      <c r="Q317" t="n">
+        <v>7237.635066215625</v>
+      </c>
+      <c r="R317" t="n">
+        <v>0</v>
+      </c>
+      <c r="S317" t="n">
+        <v>0</v>
+      </c>
+      <c r="T317" t="n">
+        <v>0</v>
+      </c>
+      <c r="U317" t="n">
+        <v>8.209569775222587</v>
+      </c>
+      <c r="V317" t="n">
+        <v>20.2590000629425</v>
+      </c>
+      <c r="W317" t="n">
+        <v>73544992.036966</v>
+      </c>
+      <c r="X317" t="n">
+        <v>73544992.036966</v>
+      </c>
+      <c r="Y317" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z317" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA317" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB317" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC317" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD317" t="inlineStr">
+        <is>
+          <t>carbon_tax_200_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE317" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260806120408_carbon_tax_200_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="n">
+        <v>79418380.06508745</v>
+      </c>
+      <c r="B318" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C318" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="D318" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E318" t="n">
+        <v>0</v>
+      </c>
+      <c r="F318" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G318" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="H318" t="n">
+        <v>25929944.4369162</v>
+      </c>
+      <c r="I318" t="n">
+        <v>0</v>
+      </c>
+      <c r="J318" t="n">
+        <v>0</v>
+      </c>
+      <c r="K318" t="n">
+        <v>0</v>
+      </c>
+      <c r="L318" t="n">
+        <v>1447527.013243193</v>
+      </c>
+      <c r="M318" t="n">
+        <v>79418380.06508745</v>
+      </c>
+      <c r="N318" t="n">
+        <v>7245.844635991023</v>
+      </c>
+      <c r="O318" t="n">
+        <v>0</v>
+      </c>
+      <c r="P318" t="n">
+        <v>7245.844635991023</v>
+      </c>
+      <c r="Q318" t="n">
+        <v>7237.635066215884</v>
+      </c>
+      <c r="R318" t="n">
+        <v>0</v>
+      </c>
+      <c r="S318" t="n">
+        <v>0</v>
+      </c>
+      <c r="T318" t="n">
+        <v>0</v>
+      </c>
+      <c r="U318" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V318" t="n">
+        <v>17.33299994468689</v>
+      </c>
+      <c r="W318" t="n">
+        <v>79418380.06508745</v>
+      </c>
+      <c r="X318" t="n">
+        <v>79418380.06508745</v>
+      </c>
+      <c r="Y318" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z318" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA318" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB318" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC318" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD318" t="inlineStr">
+        <is>
+          <t>carbon_tax_200_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE318" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260806120936_carbon_tax_200_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="n">
+        <v>85291768.09320898</v>
+      </c>
+      <c r="B319" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C319" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="D319" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E319" t="n">
+        <v>0</v>
+      </c>
+      <c r="F319" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G319" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="H319" t="n">
+        <v>31803332.46503772</v>
+      </c>
+      <c r="I319" t="n">
+        <v>0</v>
+      </c>
+      <c r="J319" t="n">
+        <v>0</v>
+      </c>
+      <c r="K319" t="n">
+        <v>0</v>
+      </c>
+      <c r="L319" t="n">
+        <v>1447527.013243193</v>
+      </c>
+      <c r="M319" t="n">
+        <v>85291768.09320898</v>
+      </c>
+      <c r="N319" t="n">
+        <v>7245.844635991023</v>
+      </c>
+      <c r="O319" t="n">
+        <v>0</v>
+      </c>
+      <c r="P319" t="n">
+        <v>7245.844635991023</v>
+      </c>
+      <c r="Q319" t="n">
+        <v>7237.635066215884</v>
+      </c>
+      <c r="R319" t="n">
+        <v>0</v>
+      </c>
+      <c r="S319" t="n">
+        <v>0</v>
+      </c>
+      <c r="T319" t="n">
+        <v>0</v>
+      </c>
+      <c r="U319" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V319" t="n">
+        <v>17.69900012016296</v>
+      </c>
+      <c r="W319" t="n">
+        <v>85291768.09320898</v>
+      </c>
+      <c r="X319" t="n">
+        <v>85291768.09320898</v>
+      </c>
+      <c r="Y319" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z319" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA319" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB319" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC319" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD319" t="inlineStr">
+        <is>
+          <t>carbon_tax_200_el_price_250</t>
+        </is>
+      </c>
+      <c r="AE319" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260806121233_carbon_tax_200_el_price_250</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="n">
+        <v>62160097.73403372</v>
+      </c>
+      <c r="B320" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C320" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="D320" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E320" t="n">
+        <v>0</v>
+      </c>
+      <c r="F320" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G320" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="H320" t="n">
+        <v>8309780.352551687</v>
+      </c>
+      <c r="I320" t="n">
+        <v>0</v>
+      </c>
+      <c r="J320" t="n">
+        <v>0</v>
+      </c>
+      <c r="K320" t="n">
+        <v>0</v>
+      </c>
+      <c r="L320" t="n">
+        <v>1809408.766553981</v>
+      </c>
+      <c r="M320" t="n">
+        <v>62160097.73403372</v>
+      </c>
+      <c r="N320" t="n">
+        <v>7245.844635991138</v>
+      </c>
+      <c r="O320" t="n">
+        <v>0</v>
+      </c>
+      <c r="P320" t="n">
+        <v>7245.844635991138</v>
+      </c>
+      <c r="Q320" t="n">
+        <v>7237.635066215954</v>
+      </c>
+      <c r="R320" t="n">
+        <v>0</v>
+      </c>
+      <c r="S320" t="n">
+        <v>0</v>
+      </c>
+      <c r="T320" t="n">
+        <v>0</v>
+      </c>
+      <c r="U320" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V320" t="n">
+        <v>16.94199991226196</v>
+      </c>
+      <c r="W320" t="n">
+        <v>62160097.73403372</v>
+      </c>
+      <c r="X320" t="n">
+        <v>62160097.73403372</v>
+      </c>
+      <c r="Y320" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z320" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA320" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB320" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC320" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD320" t="inlineStr">
+        <is>
+          <t>carbon_tax_250_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE320" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260806121527_carbon_tax_250_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="n">
+        <v>68033485.76215523</v>
+      </c>
+      <c r="B321" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C321" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="D321" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E321" t="n">
+        <v>0</v>
+      </c>
+      <c r="F321" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G321" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="H321" t="n">
+        <v>14183168.38067319</v>
+      </c>
+      <c r="I321" t="n">
+        <v>0</v>
+      </c>
+      <c r="J321" t="n">
+        <v>0</v>
+      </c>
+      <c r="K321" t="n">
+        <v>0</v>
+      </c>
+      <c r="L321" t="n">
+        <v>1809408.766553986</v>
+      </c>
+      <c r="M321" t="n">
+        <v>68033485.76215523</v>
+      </c>
+      <c r="N321" t="n">
+        <v>7245.844635991152</v>
+      </c>
+      <c r="O321" t="n">
+        <v>0</v>
+      </c>
+      <c r="P321" t="n">
+        <v>7245.844635991152</v>
+      </c>
+      <c r="Q321" t="n">
+        <v>7237.635066215976</v>
+      </c>
+      <c r="R321" t="n">
+        <v>0</v>
+      </c>
+      <c r="S321" t="n">
+        <v>0</v>
+      </c>
+      <c r="T321" t="n">
+        <v>0</v>
+      </c>
+      <c r="U321" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V321" t="n">
+        <v>18.97000002861023</v>
+      </c>
+      <c r="W321" t="n">
+        <v>68033485.76215523</v>
+      </c>
+      <c r="X321" t="n">
+        <v>68033485.76215523</v>
+      </c>
+      <c r="Y321" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z321" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA321" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB321" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC321" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD321" t="inlineStr">
+        <is>
+          <t>carbon_tax_250_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE321" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260806122109_carbon_tax_250_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="n">
+        <v>73906873.79027681</v>
+      </c>
+      <c r="B322" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C322" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="D322" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E322" t="n">
+        <v>0</v>
+      </c>
+      <c r="F322" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G322" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="H322" t="n">
+        <v>20056556.40879477</v>
+      </c>
+      <c r="I322" t="n">
+        <v>0</v>
+      </c>
+      <c r="J322" t="n">
+        <v>0</v>
+      </c>
+      <c r="K322" t="n">
+        <v>0</v>
+      </c>
+      <c r="L322" t="n">
+        <v>1809408.766553989</v>
+      </c>
+      <c r="M322" t="n">
+        <v>73906873.79027681</v>
+      </c>
+      <c r="N322" t="n">
+        <v>7245.844635991162</v>
+      </c>
+      <c r="O322" t="n">
+        <v>0</v>
+      </c>
+      <c r="P322" t="n">
+        <v>7245.844635991162</v>
+      </c>
+      <c r="Q322" t="n">
+        <v>7237.635066215978</v>
+      </c>
+      <c r="R322" t="n">
+        <v>0</v>
+      </c>
+      <c r="S322" t="n">
+        <v>0</v>
+      </c>
+      <c r="T322" t="n">
+        <v>0</v>
+      </c>
+      <c r="U322" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V322" t="n">
+        <v>19.23600006103516</v>
+      </c>
+      <c r="W322" t="n">
+        <v>73906873.79027681</v>
+      </c>
+      <c r="X322" t="n">
+        <v>73906873.79027681</v>
+      </c>
+      <c r="Y322" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z322" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA322" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB322" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC322" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD322" t="inlineStr">
+        <is>
+          <t>carbon_tax_250_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE322" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260806122403_carbon_tax_250_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="n">
+        <v>79780261.81839819</v>
+      </c>
+      <c r="B323" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C323" t="n">
+        <v>6725637.34634771</v>
+      </c>
+      <c r="D323" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E323" t="n">
+        <v>0</v>
+      </c>
+      <c r="F323" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G323" t="n">
+        <v>6725637.34634771</v>
+      </c>
+      <c r="H323" t="n">
+        <v>25929944.43691621</v>
+      </c>
+      <c r="I323" t="n">
+        <v>0</v>
+      </c>
+      <c r="J323" t="n">
+        <v>0</v>
+      </c>
+      <c r="K323" t="n">
+        <v>0</v>
+      </c>
+      <c r="L323" t="n">
+        <v>1809408.766553928</v>
+      </c>
+      <c r="M323" t="n">
+        <v>79780261.81839819</v>
+      </c>
+      <c r="N323" t="n">
+        <v>7245.84463599103</v>
+      </c>
+      <c r="O323" t="n">
+        <v>0</v>
+      </c>
+      <c r="P323" t="n">
+        <v>7245.84463599103</v>
+      </c>
+      <c r="Q323" t="n">
+        <v>7237.635066215646</v>
+      </c>
+      <c r="R323" t="n">
+        <v>0</v>
+      </c>
+      <c r="S323" t="n">
+        <v>0</v>
+      </c>
+      <c r="T323" t="n">
+        <v>0</v>
+      </c>
+      <c r="U323" t="n">
+        <v>8.209569775222587</v>
+      </c>
+      <c r="V323" t="n">
+        <v>18.83899998664856</v>
+      </c>
+      <c r="W323" t="n">
+        <v>79780261.81839819</v>
+      </c>
+      <c r="X323" t="n">
+        <v>79780261.81839819</v>
+      </c>
+      <c r="Y323" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z323" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA323" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB323" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC323" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD323" t="inlineStr">
+        <is>
+          <t>carbon_tax_250_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE323" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260806122659_carbon_tax_250_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="n">
+        <v>85653649.84651974</v>
+      </c>
+      <c r="B324" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C324" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="D324" t="n">
+        <v>27669896.37568577</v>
+      </c>
+      <c r="E324" t="n">
+        <v>0</v>
+      </c>
+      <c r="F324" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G324" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="H324" t="n">
+        <v>31803332.46503771</v>
+      </c>
+      <c r="I324" t="n">
+        <v>0</v>
+      </c>
+      <c r="J324" t="n">
+        <v>0</v>
+      </c>
+      <c r="K324" t="n">
+        <v>0</v>
+      </c>
+      <c r="L324" t="n">
+        <v>1809408.766553953</v>
+      </c>
+      <c r="M324" t="n">
+        <v>85653649.84651974</v>
+      </c>
+      <c r="N324" t="n">
+        <v>7245.844635991023</v>
+      </c>
+      <c r="O324" t="n">
+        <v>0</v>
+      </c>
+      <c r="P324" t="n">
+        <v>7245.844635991023</v>
+      </c>
+      <c r="Q324" t="n">
+        <v>7237.635066215884</v>
+      </c>
+      <c r="R324" t="n">
+        <v>0</v>
+      </c>
+      <c r="S324" t="n">
+        <v>0</v>
+      </c>
+      <c r="T324" t="n">
+        <v>0</v>
+      </c>
+      <c r="U324" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V324" t="n">
+        <v>21.21299982070923</v>
+      </c>
+      <c r="W324" t="n">
+        <v>85653649.84651974</v>
+      </c>
+      <c r="X324" t="n">
+        <v>85653649.84651974</v>
+      </c>
+      <c r="Y324" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z324" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA324" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB324" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC324" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD324" t="inlineStr">
+        <is>
+          <t>carbon_tax_250_el_price_250</t>
+        </is>
+      </c>
+      <c r="AE324" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260806122949_carbon_tax_250_el_price_250</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="n">
+        <v>62521979.48734455</v>
+      </c>
+      <c r="B325" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C325" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="D325" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E325" t="n">
+        <v>0</v>
+      </c>
+      <c r="F325" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G325" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="H325" t="n">
+        <v>8309780.352551687</v>
+      </c>
+      <c r="I325" t="n">
+        <v>0</v>
+      </c>
+      <c r="J325" t="n">
+        <v>0</v>
+      </c>
+      <c r="K325" t="n">
+        <v>0</v>
+      </c>
+      <c r="L325" t="n">
+        <v>2171290.519864807</v>
+      </c>
+      <c r="M325" t="n">
+        <v>62521979.48734455</v>
+      </c>
+      <c r="N325" t="n">
+        <v>7245.844635991085</v>
+      </c>
+      <c r="O325" t="n">
+        <v>0</v>
+      </c>
+      <c r="P325" t="n">
+        <v>7245.844635991085</v>
+      </c>
+      <c r="Q325" t="n">
+        <v>7237.635066215924</v>
+      </c>
+      <c r="R325" t="n">
+        <v>0</v>
+      </c>
+      <c r="S325" t="n">
+        <v>0</v>
+      </c>
+      <c r="T325" t="n">
+        <v>0</v>
+      </c>
+      <c r="U325" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V325" t="n">
+        <v>18.89400005340576</v>
+      </c>
+      <c r="W325" t="n">
+        <v>62521979.48732942</v>
+      </c>
+      <c r="X325" t="n">
+        <v>62521979.48734455</v>
+      </c>
+      <c r="Y325" t="n">
+        <v>1.512467861175537e-05</v>
+      </c>
+      <c r="Z325" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA325" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB325" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC325" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD325" t="inlineStr">
+        <is>
+          <t>carbon_tax_300_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE325" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260806123642_carbon_tax_300_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="n">
+        <v>68395367.51546606</v>
+      </c>
+      <c r="B326" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C326" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="D326" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E326" t="n">
+        <v>0</v>
+      </c>
+      <c r="F326" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G326" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="H326" t="n">
+        <v>14183168.38067319</v>
+      </c>
+      <c r="I326" t="n">
+        <v>0</v>
+      </c>
+      <c r="J326" t="n">
+        <v>0</v>
+      </c>
+      <c r="K326" t="n">
+        <v>0</v>
+      </c>
+      <c r="L326" t="n">
+        <v>2171290.519864818</v>
+      </c>
+      <c r="M326" t="n">
+        <v>68395367.51546606</v>
+      </c>
+      <c r="N326" t="n">
+        <v>7245.844635991118</v>
+      </c>
+      <c r="O326" t="n">
+        <v>0</v>
+      </c>
+      <c r="P326" t="n">
+        <v>7245.844635991118</v>
+      </c>
+      <c r="Q326" t="n">
+        <v>7237.63506621595</v>
+      </c>
+      <c r="R326" t="n">
+        <v>0</v>
+      </c>
+      <c r="S326" t="n">
+        <v>0</v>
+      </c>
+      <c r="T326" t="n">
+        <v>0</v>
+      </c>
+      <c r="U326" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V326" t="n">
+        <v>18.96300005912781</v>
+      </c>
+      <c r="W326" t="n">
+        <v>68395367.51545101</v>
+      </c>
+      <c r="X326" t="n">
+        <v>68395367.51546606</v>
+      </c>
+      <c r="Y326" t="n">
+        <v>1.505017280578613e-05</v>
+      </c>
+      <c r="Z326" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA326" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB326" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC326" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD326" t="inlineStr">
+        <is>
+          <t>carbon_tax_300_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE326" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260806123937_carbon_tax_300_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="n">
+        <v>74268755.54358758</v>
+      </c>
+      <c r="B327" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C327" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="D327" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E327" t="n">
+        <v>0</v>
+      </c>
+      <c r="F327" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G327" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="H327" t="n">
+        <v>20056556.40879477</v>
+      </c>
+      <c r="I327" t="n">
+        <v>0</v>
+      </c>
+      <c r="J327" t="n">
+        <v>0</v>
+      </c>
+      <c r="K327" t="n">
+        <v>0</v>
+      </c>
+      <c r="L327" t="n">
+        <v>2171290.519864755</v>
+      </c>
+      <c r="M327" t="n">
+        <v>74268755.54358758</v>
+      </c>
+      <c r="N327" t="n">
+        <v>7245.844635991075</v>
+      </c>
+      <c r="O327" t="n">
+        <v>0</v>
+      </c>
+      <c r="P327" t="n">
+        <v>7245.844635991075</v>
+      </c>
+      <c r="Q327" t="n">
+        <v>7237.635066215767</v>
+      </c>
+      <c r="R327" t="n">
+        <v>0</v>
+      </c>
+      <c r="S327" t="n">
+        <v>0</v>
+      </c>
+      <c r="T327" t="n">
+        <v>0</v>
+      </c>
+      <c r="U327" t="n">
+        <v>8.209569775222585</v>
+      </c>
+      <c r="V327" t="n">
+        <v>19.77199983596802</v>
+      </c>
+      <c r="W327" t="n">
+        <v>74268755.54357257</v>
+      </c>
+      <c r="X327" t="n">
+        <v>74268755.54358758</v>
+      </c>
+      <c r="Y327" t="n">
+        <v>1.500546932220459e-05</v>
+      </c>
+      <c r="Z327" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA327" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB327" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC327" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD327" t="inlineStr">
+        <is>
+          <t>carbon_tax_300_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE327" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260806124232_carbon_tax_300_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="n">
+        <v>80142143.57170908</v>
+      </c>
+      <c r="B328" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C328" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="D328" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E328" t="n">
+        <v>0</v>
+      </c>
+      <c r="F328" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G328" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="H328" t="n">
+        <v>25929944.4369162</v>
+      </c>
+      <c r="I328" t="n">
+        <v>0</v>
+      </c>
+      <c r="J328" t="n">
+        <v>0</v>
+      </c>
+      <c r="K328" t="n">
+        <v>0</v>
+      </c>
+      <c r="L328" t="n">
+        <v>2171290.519864826</v>
+      </c>
+      <c r="M328" t="n">
+        <v>80142143.57170908</v>
+      </c>
+      <c r="N328" t="n">
+        <v>7245.844635991145</v>
+      </c>
+      <c r="O328" t="n">
+        <v>0</v>
+      </c>
+      <c r="P328" t="n">
+        <v>7245.844635991145</v>
+      </c>
+      <c r="Q328" t="n">
+        <v>7237.635066215958</v>
+      </c>
+      <c r="R328" t="n">
+        <v>0</v>
+      </c>
+      <c r="S328" t="n">
+        <v>0</v>
+      </c>
+      <c r="T328" t="n">
+        <v>0</v>
+      </c>
+      <c r="U328" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V328" t="n">
+        <v>20.25</v>
+      </c>
+      <c r="W328" t="n">
+        <v>80142143.57169427</v>
+      </c>
+      <c r="X328" t="n">
+        <v>80142143.57170908</v>
+      </c>
+      <c r="Y328" t="n">
+        <v>1.481175422668457e-05</v>
+      </c>
+      <c r="Z328" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA328" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB328" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC328" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD328" t="inlineStr">
+        <is>
+          <t>carbon_tax_300_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE328" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260806124528_carbon_tax_300_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="n">
+        <v>86015531.59983046</v>
+      </c>
+      <c r="B329" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C329" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="D329" t="n">
+        <v>27669896.37568576</v>
+      </c>
+      <c r="E329" t="n">
+        <v>0</v>
+      </c>
+      <c r="F329" t="n">
+        <v>45315271.26858035</v>
+      </c>
+      <c r="G329" t="n">
+        <v>6725637.346347707</v>
+      </c>
+      <c r="H329" t="n">
+        <v>31803332.46503773</v>
+      </c>
+      <c r="I329" t="n">
+        <v>0</v>
+      </c>
+      <c r="J329" t="n">
+        <v>0</v>
+      </c>
+      <c r="K329" t="n">
+        <v>0</v>
+      </c>
+      <c r="L329" t="n">
+        <v>2171290.519864698</v>
+      </c>
+      <c r="M329" t="n">
+        <v>86015531.59983046</v>
+      </c>
+      <c r="N329" t="n">
+        <v>7245.84463599103</v>
+      </c>
+      <c r="O329" t="n">
+        <v>0</v>
+      </c>
+      <c r="P329" t="n">
+        <v>7245.84463599103</v>
+      </c>
+      <c r="Q329" t="n">
+        <v>7237.635066215632</v>
+      </c>
+      <c r="R329" t="n">
+        <v>0</v>
+      </c>
+      <c r="S329" t="n">
+        <v>0</v>
+      </c>
+      <c r="T329" t="n">
+        <v>0</v>
+      </c>
+      <c r="U329" t="n">
+        <v>8.209569775222587</v>
+      </c>
+      <c r="V329" t="n">
+        <v>20.41899991035461</v>
+      </c>
+      <c r="W329" t="n">
+        <v>86015531.59981579</v>
+      </c>
+      <c r="X329" t="n">
+        <v>86015531.59983046</v>
+      </c>
+      <c r="Y329" t="n">
+        <v>1.467764377593994e-05</v>
+      </c>
+      <c r="Z329" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA329" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB329" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC329" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD329" t="inlineStr">
+        <is>
+          <t>carbon_tax_300_el_price_250</t>
+        </is>
+      </c>
+      <c r="AE329" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\tech_selection\20260806125316_carbon_tax_300_el_price_250</t>
         </is>
       </c>
     </row>

</xml_diff>